<commit_message>
publish pork retail Excel 2026-07-23
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-07-22</t>
+          <t>越南猪肉零售价格日报｜2026-07-23</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 09:39。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 07:58。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,12 +588,12 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>11条在售商品</t>
+          <t>9条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>渠道：Bách Hóa Xanh、Kingfoodmart</t>
+          <t>渠道：Kingfoodmart、WinMart</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>BAF、C.P.、Meatcool、Vĩnh Tân</t>
+          <t>BAF、MEATDeli、Meatcool、Vĩnh Tân</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -632,7 +632,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>8组</t>
+          <t>13组</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-07-22</t>
+          <t>越南猪肉零售明细｜2026-07-23</t>
         </is>
       </c>
     </row>
@@ -812,32 +812,32 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Bách Hóa Xanh默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Bách Hóa Xanh</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>C.P. Vietnam</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>C.P.</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>五花肉</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Ba rọi heo giá tốt tại Bách hoá XANH</t>
+          <t>Nạc dăm heo Meatcool 360-440g</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -846,27 +846,29 @@
         </is>
       </c>
       <c r="I5" s="7" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>51000</v>
+        <v>90400</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>170000</v>
-      </c>
-      <c r="L5" s="7" t="n"/>
+        <v>226000</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <v>192100</v>
+      </c>
       <c r="M5" s="7">
         <f>IF(L5&lt;&gt;"",L5,K5)</f>
         <v/>
       </c>
       <c r="N5" s="5" t="inlineStr">
         <is>
-          <t>中：交易页价格有效期为当天，但尚未固定配送门店且原价未展示</t>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
         </is>
       </c>
       <c r="O5" s="8" t="inlineStr">
         <is>
-          <t>https://www.bachhoaxanh.com/thit-heo/ba-roi-heo</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-meatcool-400g</t>
         </is>
       </c>
     </row>
@@ -878,32 +880,32 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Bách Hóa Xanh默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Bách Hóa Xanh</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>C.P. Vietnam</t>
+          <t>BAF</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>C.P.</t>
+          <t>BAF</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>去肋五花肉</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Ba rọi heo rút sườn C.P khay 300g giá tốt tại Bách hoá XANH</t>
+          <t>Nạc dăm heo BAF khay 300g</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -915,10 +917,10 @@
         <v>300</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>80000</v>
+        <v>74000</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>266667</v>
+        <v>246667</v>
       </c>
       <c r="L6" s="7" t="n"/>
       <c r="M6" s="7">
@@ -927,12 +929,12 @@
       </c>
       <c r="N6" s="5" t="inlineStr">
         <is>
-          <t>中：交易页价格有效期为当天，但尚未固定配送门店且原价未展示</t>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
         </is>
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
-          <t>https://www.bachhoaxanh.com/thit-heo/ba-roi-heo-rut-suon-cp-khay-300g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
         </is>
       </c>
     </row>
@@ -944,32 +946,32 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Bách Hóa Xanh默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Bách Hóa Xanh</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>C.P. Vietnam</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>C.P.</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Thịt đùi heo 300g giá tốt tại Bách hoá XANH</t>
+          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -978,13 +980,13 @@
         </is>
       </c>
       <c r="I7" s="7" t="n">
-        <v>300</v>
+        <v>900</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>39000</v>
+        <v>125000</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>130000</v>
+        <v>138889</v>
       </c>
       <c r="L7" s="7" t="n"/>
       <c r="M7" s="7">
@@ -993,12 +995,12 @@
       </c>
       <c r="N7" s="5" t="inlineStr">
         <is>
-          <t>中：交易页价格有效期为当天，但尚未固定配送门店且原价未展示</t>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
         </is>
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>https://www.bachhoaxanh.com/thit-heo/thit-dui-heo-300g</t>
+          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -1010,32 +1012,32 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Bách Hóa Xanh默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Bách Hóa Xanh</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>C.P. Vietnam</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>C.P.</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>猪瘦肉</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Thịt nạc heo tại Bách hoá XANH</t>
+          <t>Thịt đùi Meatcool túi 900g</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1044,13 +1046,13 @@
         </is>
       </c>
       <c r="I8" s="7" t="n">
-        <v>300</v>
+        <v>900</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>42000</v>
+        <v>125000</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>140000</v>
+        <v>138889</v>
       </c>
       <c r="L8" s="7" t="n"/>
       <c r="M8" s="7">
@@ -1059,12 +1061,12 @@
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>中：交易页价格有效期为当天，但尚未固定配送门店且原价未展示</t>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
         </is>
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://www.bachhoaxanh.com/thit-heo/thit-nac-heo-300g</t>
+          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -1086,12 +1088,12 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -1101,7 +1103,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Meatcool 360-440g</t>
+          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1110,17 +1112,15 @@
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>90400</v>
+        <v>38000</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>226000</v>
-      </c>
-      <c r="L9" s="7" t="n">
-        <v>192100</v>
-      </c>
+        <v>190000</v>
+      </c>
+      <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
         <f>IF(L9&lt;&gt;"",L9,K9)</f>
         <v/>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-meatcool-400g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
@@ -1154,22 +1154,22 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>BAF</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>BAF</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo BAF khay 300g</t>
+          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -1178,13 +1178,13 @@
         </is>
       </c>
       <c r="I10" s="7" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>74000</v>
+        <v>79000</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>246667</v>
+        <v>197500</v>
       </c>
       <c r="L10" s="7" t="n"/>
       <c r="M10" s="7">
@@ -1198,7 +1198,7 @@
       </c>
       <c r="O10" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
         </is>
       </c>
     </row>
@@ -1220,22 +1220,22 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
+          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1244,13 +1244,13 @@
         </is>
       </c>
       <c r="I11" s="7" t="n">
-        <v>900</v>
+        <v>200</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>125000</v>
+        <v>33000</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>138889</v>
+        <v>165000</v>
       </c>
       <c r="L11" s="7" t="n"/>
       <c r="M11" s="7">
@@ -1264,44 +1264,44 @@
       </c>
       <c r="O11" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>小排</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Thịt đùi Meatcool túi 900g</t>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1310,13 +1310,13 @@
         </is>
       </c>
       <c r="I12" s="7" t="n">
-        <v>900</v>
+        <v>431</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>125000</v>
+        <v>124085</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>138889</v>
+        <v>287900</v>
       </c>
       <c r="L12" s="7" t="n"/>
       <c r="M12" s="7">
@@ -1325,49 +1325,49 @@
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O12" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -1376,13 +1376,13 @@
         </is>
       </c>
       <c r="I13" s="7" t="n">
-        <v>200</v>
+        <v>385</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>37000</v>
+        <v>76962</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>185000</v>
+        <v>199900</v>
       </c>
       <c r="L13" s="7" t="n"/>
       <c r="M13" s="7">
@@ -1391,144 +1391,12 @@
       </c>
       <c r="N13" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O13" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>南部</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Kingfoodmart</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Vĩnh Tân</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>Vĩnh Tân</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>猪排</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I14" s="7" t="n">
-        <v>400</v>
-      </c>
-      <c r="J14" s="7" t="n">
-        <v>79000</v>
-      </c>
-      <c r="K14" s="7" t="n">
-        <v>197500</v>
-      </c>
-      <c r="L14" s="7" t="n"/>
-      <c r="M14" s="7">
-        <f>IF(L14&lt;&gt;"",L14,K14)</f>
-        <v/>
-      </c>
-      <c r="N14" s="5" t="inlineStr">
-        <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
-        </is>
-      </c>
-      <c r="O14" s="8" t="inlineStr">
-        <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>南部</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Kingfoodmart</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Vĩnh Tân</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>Vĩnh Tân</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>后腿肉</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I15" s="7" t="n">
-        <v>200</v>
-      </c>
-      <c r="J15" s="7" t="n">
-        <v>33000</v>
-      </c>
-      <c r="K15" s="7" t="n">
-        <v>165000</v>
-      </c>
-      <c r="L15" s="7" t="n"/>
-      <c r="M15" s="7">
-        <f>IF(L15&lt;&gt;"",L15,K15)</f>
-        <v/>
-      </c>
-      <c r="N15" s="5" t="inlineStr">
-        <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
-        </is>
-      </c>
-      <c r="O15" s="8" t="inlineStr">
-        <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
+          <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
       </c>
     </row>
@@ -1537,7 +1405,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M15">
+  <conditionalFormatting sqref="M5:M13">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1555,8 +1423,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1671,7 +1537,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1881,7 +1747,7 @@
         </is>
       </c>
       <c r="E10" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" s="7" t="n">
         <v>199900</v>
@@ -1923,7 +1789,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>287900</v>
@@ -2049,7 +1915,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>138889</v>
@@ -2091,7 +1957,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>226000</v>
@@ -2100,7 +1966,7 @@
         <v>192100</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>209050</v>
+        <v>192100</v>
       </c>
       <c r="I15" s="9">
         <f>IF(E15&lt;2,"",G15/F15-1)</f>
@@ -2133,7 +1999,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>138889</v>
@@ -2175,7 +2041,7 @@
         </is>
       </c>
       <c r="E17" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F17" s="7" t="n">
         <v>165000</v>
@@ -2217,16 +2083,16 @@
         </is>
       </c>
       <c r="E18" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F18" s="7" t="n">
         <v>185000</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>185000</v>
+        <v>190000</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>185000</v>
+        <v>187500</v>
       </c>
       <c r="I18" s="9">
         <f>IF(E18&lt;2,"",G18/F18-1)</f>
@@ -2259,7 +2125,7 @@
         </is>
       </c>
       <c r="E19" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F19" s="7" t="n">
         <v>197500</v>
@@ -2362,12 +2228,12 @@
     <row r="5" ht="58" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Bách Hóa Xanh</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>C.P. Vietnam / C.P.</t>
+          <t>GREENFEED / Meatcool</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -2382,12 +2248,12 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>中：交易页价格有效期为当天，但尚未固定配送门店且原价未展示</t>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>https://www.bachhoaxanh.com/thit-heo/ba-roi-heo</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-meatcool-400g</t>
         </is>
       </c>
     </row>
@@ -2399,7 +2265,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED / Meatcool</t>
+          <t>BAF / BAF</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -2419,7 +2285,7 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-meatcool-400g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
         </is>
       </c>
     </row>
@@ -2431,7 +2297,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>BAF / BAF</t>
+          <t>Vĩnh Tân / Vĩnh Tân</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -2451,24 +2317,24 @@
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
     <row r="8" ht="58" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân / Vĩnh Tân</t>
+          <t>Masan / MEATDeli</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>A-零售交易页</t>
+          <t>A-官方交易页</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -2478,12 +2344,12 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-07-24
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-07-24</t>
+          <t>越南猪肉零售价格日报｜2026-07-25</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 05:38。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 05:43。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>9条在售商品</t>
+          <t>7条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -610,12 +610,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>4个</t>
+          <t>3个</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>BAF、MEATDeli、Meatcool、Vĩnh Tân</t>
+          <t>MEATDeli、Meatcool、Vĩnh Tân</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -632,7 +632,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>13组</t>
+          <t>14组</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:O11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-07-24</t>
+          <t>越南猪肉零售明细｜2026-07-25</t>
         </is>
       </c>
     </row>
@@ -854,9 +854,7 @@
       <c r="K5" s="7" t="n">
         <v>226000</v>
       </c>
-      <c r="L5" s="7" t="n">
-        <v>192100</v>
-      </c>
+      <c r="L5" s="7" t="n"/>
       <c r="M5" s="7">
         <f>IF(L5&lt;&gt;"",L5,K5)</f>
         <v/>
@@ -890,22 +888,22 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>BAF</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>BAF</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo BAF khay 300g</t>
+          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -914,13 +912,13 @@
         </is>
       </c>
       <c r="I6" s="7" t="n">
-        <v>300</v>
+        <v>900</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>74000</v>
+        <v>125000</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>246667</v>
+        <v>138889</v>
       </c>
       <c r="L6" s="7" t="n"/>
       <c r="M6" s="7">
@@ -934,7 +932,7 @@
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -966,12 +964,12 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
+          <t>Thịt đùi Meatcool túi 900g</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -1000,7 +998,7 @@
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -1022,22 +1020,22 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Thịt đùi Meatcool túi 900g</t>
+          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1046,13 +1044,13 @@
         </is>
       </c>
       <c r="I8" s="7" t="n">
-        <v>900</v>
+        <v>400</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>125000</v>
+        <v>79000</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>138889</v>
+        <v>197500</v>
       </c>
       <c r="L8" s="7" t="n"/>
       <c r="M8" s="7">
@@ -1066,44 +1064,44 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
         </is>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>小排</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1112,13 +1110,13 @@
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>200</v>
+        <v>431</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>38000</v>
+        <v>124085</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>190000</v>
+        <v>287900</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
@@ -1127,49 +1125,49 @@
       </c>
       <c r="N9" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
+          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -1181,10 +1179,10 @@
         <v>400</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>79000</v>
+        <v>81960</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>197500</v>
+        <v>204900</v>
       </c>
       <c r="L10" s="7" t="n"/>
       <c r="M10" s="7">
@@ -1193,49 +1191,49 @@
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O10" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
+          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
         </is>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1244,13 +1242,13 @@
         </is>
       </c>
       <c r="I11" s="7" t="n">
-        <v>200</v>
+        <v>385</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>33000</v>
+        <v>76962</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>165000</v>
+        <v>199900</v>
       </c>
       <c r="L11" s="7" t="n"/>
       <c r="M11" s="7">
@@ -1259,142 +1257,10 @@
       </c>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O11" s="8" t="inlineStr">
-        <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>小排</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I12" s="7" t="n">
-        <v>431</v>
-      </c>
-      <c r="J12" s="7" t="n">
-        <v>124085</v>
-      </c>
-      <c r="K12" s="7" t="n">
-        <v>287900</v>
-      </c>
-      <c r="L12" s="7" t="n"/>
-      <c r="M12" s="7">
-        <f>IF(L12&lt;&gt;"",L12,K12)</f>
-        <v/>
-      </c>
-      <c r="N12" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O12" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>五花肉</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I13" s="7" t="n">
-        <v>385</v>
-      </c>
-      <c r="J13" s="7" t="n">
-        <v>76962</v>
-      </c>
-      <c r="K13" s="7" t="n">
-        <v>199900</v>
-      </c>
-      <c r="L13" s="7" t="n"/>
-      <c r="M13" s="7">
-        <f>IF(L13&lt;&gt;"",L13,K13)</f>
-        <v/>
-      </c>
-      <c r="N13" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O13" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
@@ -1405,7 +1271,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M13">
+  <conditionalFormatting sqref="M5:M11">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1421,8 +1287,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1747,7 +1611,7 @@
         </is>
       </c>
       <c r="E10" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F10" s="7" t="n">
         <v>199900</v>
@@ -1789,7 +1653,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>287900</v>
@@ -1831,7 +1695,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>204900</v>
@@ -1915,7 +1779,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>138889</v>
@@ -1957,13 +1821,13 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>226000</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>192100</v>
+        <v>226000</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>192100</v>
@@ -1999,7 +1863,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>138889</v>
@@ -2125,7 +1989,7 @@
         </is>
       </c>
       <c r="E19" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F19" s="7" t="n">
         <v>197500</v>
@@ -2168,7 +2032,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2265,7 +2129,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>BAF / BAF</t>
+          <t>Vĩnh Tân / Vĩnh Tân</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -2285,24 +2149,24 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
         </is>
       </c>
     </row>
     <row r="7" ht="58" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân / Vĩnh Tân</t>
+          <t>Masan / MEATDeli</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>A-零售交易页</t>
+          <t>A-官方交易页</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -2312,42 +2176,10 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="58" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Masan / MEATDeli</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>A-官方交易页</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>实际价/kg = 促销价/kg（如有），否则常规价/kg；包装价÷重量(kg)用于交叉核验。</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
@@ -2362,7 +2194,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-07-25
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-07-25</t>
+          <t>越南猪肉零售价格日报｜2026-07-26</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 05:43。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 05:38。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-07-25</t>
+          <t>越南猪肉零售明细｜2026-07-26</t>
         </is>
       </c>
     </row>
@@ -1611,7 +1611,7 @@
         </is>
       </c>
       <c r="E10" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F10" s="7" t="n">
         <v>199900</v>
@@ -1653,7 +1653,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>287900</v>
@@ -1695,7 +1695,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>204900</v>
@@ -1779,7 +1779,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>138889</v>
@@ -1821,7 +1821,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>226000</v>
@@ -1830,7 +1830,7 @@
         <v>226000</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>192100</v>
+        <v>209050</v>
       </c>
       <c r="I15" s="9">
         <f>IF(E15&lt;2,"",G15/F15-1)</f>
@@ -1863,7 +1863,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>138889</v>
@@ -1989,7 +1989,7 @@
         </is>
       </c>
       <c r="E19" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F19" s="7" t="n">
         <v>197500</v>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-07-26
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-07-26</t>
+          <t>越南猪肉零售价格日报｜2026-07-27</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 05:38。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 05:44。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,12 +588,12 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>7条在售商品</t>
+          <t>5条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>渠道：Kingfoodmart、WinMart</t>
+          <t>渠道：Kingfoodmart</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>MEATDeli、Meatcool、Vĩnh Tân</t>
+          <t>BAF、Meatcool、Vĩnh Tân</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:O9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-07-26</t>
+          <t>越南猪肉零售明细｜2026-07-27</t>
         </is>
       </c>
     </row>
@@ -854,7 +854,9 @@
       <c r="K5" s="7" t="n">
         <v>226000</v>
       </c>
-      <c r="L5" s="7" t="n"/>
+      <c r="L5" s="7" t="n">
+        <v>192100</v>
+      </c>
       <c r="M5" s="7">
         <f>IF(L5&lt;&gt;"",L5,K5)</f>
         <v/>
@@ -888,22 +890,22 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>BAF</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>BAF</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
+          <t>Nạc dăm heo BAF khay 300g</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -912,13 +914,13 @@
         </is>
       </c>
       <c r="I6" s="7" t="n">
-        <v>900</v>
+        <v>300</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>125000</v>
+        <v>74000</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>138889</v>
+        <v>246667</v>
       </c>
       <c r="L6" s="7" t="n"/>
       <c r="M6" s="7">
@@ -932,7 +934,7 @@
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
         </is>
       </c>
     </row>
@@ -954,22 +956,22 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Thịt đùi Meatcool túi 900g</t>
+          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -978,13 +980,13 @@
         </is>
       </c>
       <c r="I7" s="7" t="n">
-        <v>900</v>
+        <v>200</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>125000</v>
+        <v>38000</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>138889</v>
+        <v>190000</v>
       </c>
       <c r="L7" s="7" t="n"/>
       <c r="M7" s="7">
@@ -998,7 +1000,7 @@
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
@@ -1071,37 +1073,37 @@
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>全国渠道</t>
+          <t>南部</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>WinMart默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>WinMart</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Masan</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>MEATDeli</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>小排</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
+          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1110,13 +1112,13 @@
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>431</v>
+        <v>200</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>124085</v>
+        <v>33000</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>287900</v>
+        <v>165000</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
@@ -1125,144 +1127,12 @@
       </c>
       <c r="N9" s="5" t="inlineStr">
         <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
         </is>
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>梅花肉</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I10" s="7" t="n">
-        <v>400</v>
-      </c>
-      <c r="J10" s="7" t="n">
-        <v>81960</v>
-      </c>
-      <c r="K10" s="7" t="n">
-        <v>204900</v>
-      </c>
-      <c r="L10" s="7" t="n"/>
-      <c r="M10" s="7">
-        <f>IF(L10&lt;&gt;"",L10,K10)</f>
-        <v/>
-      </c>
-      <c r="N10" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O10" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>五花肉</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I11" s="7" t="n">
-        <v>385</v>
-      </c>
-      <c r="J11" s="7" t="n">
-        <v>76962</v>
-      </c>
-      <c r="K11" s="7" t="n">
-        <v>199900</v>
-      </c>
-      <c r="L11" s="7" t="n"/>
-      <c r="M11" s="7">
-        <f>IF(L11&lt;&gt;"",L11,K11)</f>
-        <v/>
-      </c>
-      <c r="N11" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O11" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1141,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M11">
+  <conditionalFormatting sqref="M5:M9">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1285,8 +1155,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1401,7 +1269,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1821,16 +1689,16 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>226000</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>226000</v>
+        <v>192100</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>209050</v>
+        <v>192100</v>
       </c>
       <c r="I15" s="9">
         <f>IF(E15&lt;2,"",G15/F15-1)</f>
@@ -1905,7 +1773,7 @@
         </is>
       </c>
       <c r="E17" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F17" s="7" t="n">
         <v>165000</v>
@@ -1947,7 +1815,7 @@
         </is>
       </c>
       <c r="E18" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F18" s="7" t="n">
         <v>185000</v>
@@ -1989,7 +1857,7 @@
         </is>
       </c>
       <c r="E19" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F19" s="7" t="n">
         <v>197500</v>
@@ -2129,7 +1997,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân / Vĩnh Tân</t>
+          <t>BAF / BAF</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -2149,24 +2017,24 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
         </is>
       </c>
     </row>
     <row r="7" ht="58" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>WinMart</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Masan / MEATDeli</t>
+          <t>Vĩnh Tân / Vĩnh Tân</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>A-官方交易页</t>
+          <t>A-零售交易页</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -2176,12 +2044,12 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-07-27
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-07-27</t>
+          <t>越南猪肉零售价格日报｜2026-07-28</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 05:44。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 05:42。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,12 +588,12 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>5条在售商品</t>
+          <t>9条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>渠道：Kingfoodmart</t>
+          <t>渠道：Kingfoodmart、WinMart</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -610,12 +610,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>3个</t>
+          <t>4个</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>BAF、Meatcool、Vĩnh Tân</t>
+          <t>BAF、MEATDeli、Meatcool、Vĩnh Tân</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O9"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-07-27</t>
+          <t>越南猪肉零售明细｜2026-07-28</t>
         </is>
       </c>
     </row>
@@ -956,22 +956,22 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
+          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -980,13 +980,13 @@
         </is>
       </c>
       <c r="I7" s="7" t="n">
-        <v>200</v>
+        <v>900</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>38000</v>
+        <v>125000</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>190000</v>
+        <v>138889</v>
       </c>
       <c r="L7" s="7" t="n"/>
       <c r="M7" s="7">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
+          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -1022,22 +1022,22 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
+          <t>Thịt đùi Meatcool túi 900g</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1046,13 +1046,13 @@
         </is>
       </c>
       <c r="I8" s="7" t="n">
-        <v>400</v>
+        <v>900</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>79000</v>
+        <v>125000</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>197500</v>
+        <v>138889</v>
       </c>
       <c r="L8" s="7" t="n"/>
       <c r="M8" s="7">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -1098,12 +1098,12 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
+          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1115,10 +1115,10 @@
         <v>200</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>33000</v>
+        <v>38000</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>165000</v>
+        <v>190000</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
@@ -1132,7 +1132,271 @@
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>南部</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>胡志明市/Kingfoodmart默认门店</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Kingfoodmart</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Vĩnh Tân</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Vĩnh Tân</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>猪排</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>冷鲜</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="n">
+        <v>400</v>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>79000</v>
+      </c>
+      <c r="K10" s="7" t="n">
+        <v>197500</v>
+      </c>
+      <c r="L10" s="7" t="n"/>
+      <c r="M10" s="7">
+        <f>IF(L10&lt;&gt;"",L10,K10)</f>
+        <v/>
+      </c>
+      <c r="N10" s="5" t="inlineStr">
+        <is>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+        </is>
+      </c>
+      <c r="O10" s="8" t="inlineStr">
+        <is>
+          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>南部</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>胡志明市/Kingfoodmart默认门店</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Kingfoodmart</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Vĩnh Tân</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Vĩnh Tân</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>后腿肉</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>冷鲜</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>33000</v>
+      </c>
+      <c r="K11" s="7" t="n">
+        <v>165000</v>
+      </c>
+      <c r="L11" s="7" t="n"/>
+      <c r="M11" s="7">
+        <f>IF(L11&lt;&gt;"",L11,K11)</f>
+        <v/>
+      </c>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+        </is>
+      </c>
+      <c r="O11" s="8" t="inlineStr">
+        <is>
           <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>全国渠道</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>WinMart默认门店（待固定城市）</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>WinMart</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Masan</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>MEATDeli</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>小排</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>冷鲜</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="n">
+        <v>431</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>124085</v>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>287900</v>
+      </c>
+      <c r="L12" s="7" t="n"/>
+      <c r="M12" s="7">
+        <f>IF(L12&lt;&gt;"",L12,K12)</f>
+        <v/>
+      </c>
+      <c r="N12" s="5" t="inlineStr">
+        <is>
+          <t>中：官方交易页，但尚未固定配送门店</t>
+        </is>
+      </c>
+      <c r="O12" s="8" t="inlineStr">
+        <is>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>全国渠道</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>WinMart默认门店（待固定城市）</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>WinMart</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Masan</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>MEATDeli</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>五花肉</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>冷鲜</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>385</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>76962</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>199900</v>
+      </c>
+      <c r="L13" s="7" t="n"/>
+      <c r="M13" s="7">
+        <f>IF(L13&lt;&gt;"",L13,K13)</f>
+        <v/>
+      </c>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>中：官方交易页，但尚未固定配送门店</t>
+        </is>
+      </c>
+      <c r="O13" s="8" t="inlineStr">
+        <is>
+          <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1405,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M9">
+  <conditionalFormatting sqref="M5:M13">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1155,6 +1419,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1269,7 +1537,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1479,7 +1747,7 @@
         </is>
       </c>
       <c r="E10" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F10" s="7" t="n">
         <v>199900</v>
@@ -1521,7 +1789,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>287900</v>
@@ -1647,7 +1915,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>138889</v>
@@ -1689,7 +1957,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>226000</v>
@@ -1731,7 +1999,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>138889</v>
@@ -1773,7 +2041,7 @@
         </is>
       </c>
       <c r="E17" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F17" s="7" t="n">
         <v>165000</v>
@@ -1815,7 +2083,7 @@
         </is>
       </c>
       <c r="E18" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F18" s="7" t="n">
         <v>185000</v>
@@ -1857,7 +2125,7 @@
         </is>
       </c>
       <c r="E19" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F19" s="7" t="n">
         <v>197500</v>
@@ -1900,7 +2168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2053,6 +2321,38 @@
         </is>
       </c>
     </row>
+    <row r="8" ht="58" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>WinMart</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Masan / MEATDeli</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>A-官方交易页</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>实际价/kg = 促销价/kg（如有），否则常规价/kg；包装价÷重量(kg)用于交叉核验。</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>中：官方交易页，但尚未固定配送门店</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
@@ -2062,6 +2362,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-07-28
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,7 +547,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-07-28</t>
+          <t>越南猪肉零售价格日报｜2026-07-29</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>9条在售商品</t>
+          <t>8条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-07-28</t>
+          <t>越南猪肉零售明细｜2026-07-29</t>
         </is>
       </c>
     </row>
@@ -1331,72 +1331,6 @@
       <c r="O12" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>五花肉</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I13" s="7" t="n">
-        <v>385</v>
-      </c>
-      <c r="J13" s="7" t="n">
-        <v>76962</v>
-      </c>
-      <c r="K13" s="7" t="n">
-        <v>199900</v>
-      </c>
-      <c r="L13" s="7" t="n"/>
-      <c r="M13" s="7">
-        <f>IF(L13&lt;&gt;"",L13,K13)</f>
-        <v/>
-      </c>
-      <c r="N13" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O13" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1339,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M13">
+  <conditionalFormatting sqref="M5:M12">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1422,7 +1356,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1537,7 +1470,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1789,7 +1722,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>287900</v>
@@ -1915,7 +1848,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>138889</v>
@@ -1957,7 +1890,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>226000</v>
@@ -1999,7 +1932,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>138889</v>
@@ -2041,7 +1974,7 @@
         </is>
       </c>
       <c r="E17" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F17" s="7" t="n">
         <v>165000</v>
@@ -2083,7 +2016,7 @@
         </is>
       </c>
       <c r="E18" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F18" s="7" t="n">
         <v>185000</v>
@@ -2125,7 +2058,7 @@
         </is>
       </c>
       <c r="E19" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F19" s="7" t="n">
         <v>197500</v>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-07-29
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-07-29</t>
+          <t>越南猪肉零售价格日报｜2026-07-30</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 05:42。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 05:39。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-07-29</t>
+          <t>越南猪肉零售明细｜2026-07-30</t>
         </is>
       </c>
     </row>
@@ -1470,7 +1470,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1722,7 +1722,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>287900</v>
@@ -1848,7 +1848,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>138889</v>
@@ -1890,7 +1890,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>226000</v>
@@ -1932,7 +1932,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>138889</v>
@@ -1974,7 +1974,7 @@
         </is>
       </c>
       <c r="E17" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F17" s="7" t="n">
         <v>165000</v>
@@ -2016,7 +2016,7 @@
         </is>
       </c>
       <c r="E18" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F18" s="7" t="n">
         <v>185000</v>
@@ -2058,7 +2058,7 @@
         </is>
       </c>
       <c r="E19" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F19" s="7" t="n">
         <v>197500</v>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-07-30
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-07-30</t>
+          <t>越南猪肉零售价格日报｜2026-07-31</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 05:39。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 05:49。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,12 +588,12 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>8条在售商品</t>
+          <t>11条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>渠道：Kingfoodmart、WinMart</t>
+          <t>渠道：Bách Hóa Xanh、Kingfoodmart</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>BAF、MEATDeli、Meatcool、Vĩnh Tân</t>
+          <t>BAF、C.P.、Meatcool、Vĩnh Tân</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O12"/>
+  <dimension ref="A1:O15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-07-30</t>
+          <t>越南猪肉零售明细｜2026-07-31</t>
         </is>
       </c>
     </row>
@@ -812,32 +812,32 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>Bách Hóa Xanh默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>Bách Hóa Xanh</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>C.P. Vietnam</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>C.P.</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Meatcool 360-440g</t>
+          <t>Ba rọi heo giá tốt tại Bách hoá XANH</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -846,29 +846,27 @@
         </is>
       </c>
       <c r="I5" s="7" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>90400</v>
+        <v>47430</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>226000</v>
-      </c>
-      <c r="L5" s="7" t="n">
-        <v>192100</v>
-      </c>
+        <v>158100</v>
+      </c>
+      <c r="L5" s="7" t="n"/>
       <c r="M5" s="7">
         <f>IF(L5&lt;&gt;"",L5,K5)</f>
         <v/>
       </c>
       <c r="N5" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：交易页价格有效期为当天，但尚未固定配送门店且原价未展示</t>
         </is>
       </c>
       <c r="O5" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-meatcool-400g</t>
+          <t>https://www.bachhoaxanh.com/thit-heo/ba-roi-heo</t>
         </is>
       </c>
     </row>
@@ -880,32 +878,32 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>Bách Hóa Xanh默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>Bách Hóa Xanh</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>BAF</t>
+          <t>C.P. Vietnam</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>BAF</t>
+          <t>C.P.</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>去肋五花肉</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo BAF khay 300g</t>
+          <t>Ba rọi heo rút sườn C.P khay 300g giá tốt tại Bách hoá XANH</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -917,10 +915,10 @@
         <v>300</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>74000</v>
+        <v>80000</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>246667</v>
+        <v>266667</v>
       </c>
       <c r="L6" s="7" t="n"/>
       <c r="M6" s="7">
@@ -929,12 +927,12 @@
       </c>
       <c r="N6" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：交易页价格有效期为当天，但尚未固定配送门店且原价未展示</t>
         </is>
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
+          <t>https://www.bachhoaxanh.com/thit-heo/ba-roi-heo-rut-suon-cp-khay-300g</t>
         </is>
       </c>
     </row>
@@ -946,32 +944,32 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>Bách Hóa Xanh默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>Bách Hóa Xanh</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>C.P. Vietnam</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>C.P.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
+          <t>Thịt đùi heo 300g giá tốt tại Bách hoá XANH</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -980,13 +978,13 @@
         </is>
       </c>
       <c r="I7" s="7" t="n">
-        <v>900</v>
+        <v>300</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>125000</v>
+        <v>34710</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>138889</v>
+        <v>115700</v>
       </c>
       <c r="L7" s="7" t="n"/>
       <c r="M7" s="7">
@@ -995,12 +993,12 @@
       </c>
       <c r="N7" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：交易页价格有效期为当天，但尚未固定配送门店且原价未展示</t>
         </is>
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
+          <t>https://www.bachhoaxanh.com/thit-heo/thit-dui-heo-300g</t>
         </is>
       </c>
     </row>
@@ -1012,32 +1010,32 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>Bách Hóa Xanh默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>Bách Hóa Xanh</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>C.P. Vietnam</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>C.P.</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>猪瘦肉</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Thịt đùi Meatcool túi 900g</t>
+          <t>Thịt nạc heo tại Bách hoá XANH</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1046,13 +1044,13 @@
         </is>
       </c>
       <c r="I8" s="7" t="n">
-        <v>900</v>
+        <v>300</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>125000</v>
+        <v>37800</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>138889</v>
+        <v>126000</v>
       </c>
       <c r="L8" s="7" t="n"/>
       <c r="M8" s="7">
@@ -1061,12 +1059,12 @@
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：交易页价格有效期为当天，但尚未固定配送门店且原价未展示</t>
         </is>
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
+          <t>https://www.bachhoaxanh.com/thit-heo/thit-nac-heo-300g</t>
         </is>
       </c>
     </row>
@@ -1088,12 +1086,12 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -1103,7 +1101,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
+          <t>Nạc dăm heo Meatcool 360-440g</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1112,15 +1110,17 @@
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>38000</v>
+        <v>90400</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>190000</v>
-      </c>
-      <c r="L9" s="7" t="n"/>
+        <v>226000</v>
+      </c>
+      <c r="L9" s="7" t="n">
+        <v>192100</v>
+      </c>
       <c r="M9" s="7">
         <f>IF(L9&lt;&gt;"",L9,K9)</f>
         <v/>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-meatcool-400g</t>
         </is>
       </c>
     </row>
@@ -1154,22 +1154,22 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>BAF</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>BAF</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
+          <t>Nạc dăm heo BAF khay 300g</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -1178,13 +1178,13 @@
         </is>
       </c>
       <c r="I10" s="7" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>79000</v>
+        <v>74000</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>197500</v>
+        <v>246667</v>
       </c>
       <c r="L10" s="7" t="n"/>
       <c r="M10" s="7">
@@ -1198,7 +1198,7 @@
       </c>
       <c r="O10" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
         </is>
       </c>
     </row>
@@ -1220,22 +1220,22 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
+          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1244,13 +1244,13 @@
         </is>
       </c>
       <c r="I11" s="7" t="n">
-        <v>200</v>
+        <v>900</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>33000</v>
+        <v>125000</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>165000</v>
+        <v>138889</v>
       </c>
       <c r="L11" s="7" t="n"/>
       <c r="M11" s="7">
@@ -1264,44 +1264,44 @@
       </c>
       <c r="O11" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
+          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>全国渠道</t>
+          <t>南部</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>WinMart默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>WinMart</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Masan</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>MEATDeli</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>小排</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
+          <t>Thịt đùi Meatcool túi 900g</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1310,13 +1310,13 @@
         </is>
       </c>
       <c r="I12" s="7" t="n">
-        <v>431</v>
+        <v>900</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>124085</v>
+        <v>125000</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>287900</v>
+        <v>138889</v>
       </c>
       <c r="L12" s="7" t="n"/>
       <c r="M12" s="7">
@@ -1325,12 +1325,210 @@
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
         </is>
       </c>
       <c r="O12" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>南部</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>胡志明市/Kingfoodmart默认门店</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Kingfoodmart</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Vĩnh Tân</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Vĩnh Tân</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>梅花肉</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>冷鲜</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>38000</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>190000</v>
+      </c>
+      <c r="L13" s="7" t="n"/>
+      <c r="M13" s="7">
+        <f>IF(L13&lt;&gt;"",L13,K13)</f>
+        <v/>
+      </c>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+        </is>
+      </c>
+      <c r="O13" s="8" t="inlineStr">
+        <is>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>南部</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>胡志明市/Kingfoodmart默认门店</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Kingfoodmart</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Vĩnh Tân</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Vĩnh Tân</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>猪排</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>冷鲜</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>400</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>79000</v>
+      </c>
+      <c r="K14" s="7" t="n">
+        <v>197500</v>
+      </c>
+      <c r="L14" s="7" t="n"/>
+      <c r="M14" s="7">
+        <f>IF(L14&lt;&gt;"",L14,K14)</f>
+        <v/>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+        </is>
+      </c>
+      <c r="O14" s="8" t="inlineStr">
+        <is>
+          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>南部</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>胡志明市/Kingfoodmart默认门店</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Kingfoodmart</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Vĩnh Tân</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Vĩnh Tân</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>后腿肉</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>冷鲜</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>33000</v>
+      </c>
+      <c r="K15" s="7" t="n">
+        <v>165000</v>
+      </c>
+      <c r="L15" s="7" t="n"/>
+      <c r="M15" s="7">
+        <f>IF(L15&lt;&gt;"",L15,K15)</f>
+        <v/>
+      </c>
+      <c r="N15" s="5" t="inlineStr">
+        <is>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+        </is>
+      </c>
+      <c r="O15" s="8" t="inlineStr">
+        <is>
+          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1537,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M12">
+  <conditionalFormatting sqref="M5:M15">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1356,6 +1554,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1470,7 +1671,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1512,16 +1713,16 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>159000</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>170000</v>
+        <v>158100</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>164500</v>
+        <v>159000</v>
       </c>
       <c r="I6" s="9">
         <f>IF(E6&lt;2,"",G6/F6-1)</f>
@@ -1554,7 +1755,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>266667</v>
@@ -1596,16 +1797,16 @@
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>109000</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>130000</v>
+        <v>115700</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>119500</v>
+        <v>115700</v>
       </c>
       <c r="I8" s="9">
         <f>IF(E8&lt;2,"",G8/F8-1)</f>
@@ -1638,16 +1839,16 @@
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>132000</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>140000</v>
+        <v>126000</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>136000</v>
+        <v>132000</v>
       </c>
       <c r="I9" s="9">
         <f>IF(E9&lt;2,"",G9/F9-1)</f>
@@ -1848,7 +2049,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>138889</v>
@@ -1890,7 +2091,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>226000</v>
@@ -1932,7 +2133,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>138889</v>
@@ -1974,7 +2175,7 @@
         </is>
       </c>
       <c r="E17" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F17" s="7" t="n">
         <v>165000</v>
@@ -2016,7 +2217,7 @@
         </is>
       </c>
       <c r="E18" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F18" s="7" t="n">
         <v>185000</v>
@@ -2058,7 +2259,7 @@
         </is>
       </c>
       <c r="E19" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F19" s="7" t="n">
         <v>197500</v>
@@ -2161,12 +2362,12 @@
     <row r="5" ht="58" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>Bách Hóa Xanh</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED / Meatcool</t>
+          <t>C.P. Vietnam / C.P.</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -2181,12 +2382,12 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：交易页价格有效期为当天，但尚未固定配送门店且原价未展示</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-meatcool-400g</t>
+          <t>https://www.bachhoaxanh.com/thit-heo/ba-roi-heo</t>
         </is>
       </c>
     </row>
@@ -2198,7 +2399,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>BAF / BAF</t>
+          <t>GREENFEED / Meatcool</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -2218,7 +2419,7 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-meatcool-400g</t>
         </is>
       </c>
     </row>
@@ -2230,7 +2431,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân / Vĩnh Tân</t>
+          <t>BAF / BAF</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -2250,24 +2451,24 @@
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
         </is>
       </c>
     </row>
     <row r="8" ht="58" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>WinMart</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Masan / MEATDeli</t>
+          <t>Vĩnh Tân / Vĩnh Tân</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>A-官方交易页</t>
+          <t>A-零售交易页</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -2277,12 +2478,12 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-07-31
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-07-31</t>
+          <t>越南猪肉零售价格日报｜2026-08-01</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 05:49。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 05:42。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,12 +588,12 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>11条在售商品</t>
+          <t>9条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>渠道：Bách Hóa Xanh、Kingfoodmart</t>
+          <t>渠道：Kingfoodmart、WinMart</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>BAF、C.P.、Meatcool、Vĩnh Tân</t>
+          <t>BAF、MEATDeli、Meatcool、Vĩnh Tân</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -632,7 +632,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>14组</t>
+          <t>0组</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-07-31</t>
+          <t>越南猪肉零售明细｜2026-08-01</t>
         </is>
       </c>
     </row>
@@ -812,32 +812,32 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Bách Hóa Xanh默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Bách Hóa Xanh</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>C.P. Vietnam</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>C.P.</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>五花肉</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Ba rọi heo giá tốt tại Bách hoá XANH</t>
+          <t>Nạc dăm heo Meatcool 360-440g</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -846,27 +846,29 @@
         </is>
       </c>
       <c r="I5" s="7" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>47430</v>
+        <v>90400</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>158100</v>
-      </c>
-      <c r="L5" s="7" t="n"/>
+        <v>226000</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <v>192100</v>
+      </c>
       <c r="M5" s="7">
         <f>IF(L5&lt;&gt;"",L5,K5)</f>
         <v/>
       </c>
       <c r="N5" s="5" t="inlineStr">
         <is>
-          <t>中：交易页价格有效期为当天，但尚未固定配送门店且原价未展示</t>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
         </is>
       </c>
       <c r="O5" s="8" t="inlineStr">
         <is>
-          <t>https://www.bachhoaxanh.com/thit-heo/ba-roi-heo</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-meatcool-400g</t>
         </is>
       </c>
     </row>
@@ -878,32 +880,32 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Bách Hóa Xanh默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Bách Hóa Xanh</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>C.P. Vietnam</t>
+          <t>BAF</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>C.P.</t>
+          <t>BAF</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>去肋五花肉</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Ba rọi heo rút sườn C.P khay 300g giá tốt tại Bách hoá XANH</t>
+          <t>Nạc dăm heo BAF khay 300g</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -915,10 +917,10 @@
         <v>300</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>80000</v>
+        <v>74000</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>266667</v>
+        <v>246667</v>
       </c>
       <c r="L6" s="7" t="n"/>
       <c r="M6" s="7">
@@ -927,12 +929,12 @@
       </c>
       <c r="N6" s="5" t="inlineStr">
         <is>
-          <t>中：交易页价格有效期为当天，但尚未固定配送门店且原价未展示</t>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
         </is>
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
-          <t>https://www.bachhoaxanh.com/thit-heo/ba-roi-heo-rut-suon-cp-khay-300g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
         </is>
       </c>
     </row>
@@ -944,32 +946,32 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Bách Hóa Xanh默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Bách Hóa Xanh</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>C.P. Vietnam</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>C.P.</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Thịt đùi heo 300g giá tốt tại Bách hoá XANH</t>
+          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -978,13 +980,13 @@
         </is>
       </c>
       <c r="I7" s="7" t="n">
-        <v>300</v>
+        <v>900</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>34710</v>
+        <v>125000</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>115700</v>
+        <v>138889</v>
       </c>
       <c r="L7" s="7" t="n"/>
       <c r="M7" s="7">
@@ -993,12 +995,12 @@
       </c>
       <c r="N7" s="5" t="inlineStr">
         <is>
-          <t>中：交易页价格有效期为当天，但尚未固定配送门店且原价未展示</t>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
         </is>
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>https://www.bachhoaxanh.com/thit-heo/thit-dui-heo-300g</t>
+          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -1010,32 +1012,32 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Bách Hóa Xanh默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Bách Hóa Xanh</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>C.P. Vietnam</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>C.P.</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>猪瘦肉</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Thịt nạc heo tại Bách hoá XANH</t>
+          <t>Thịt đùi Meatcool túi 900g</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1044,13 +1046,13 @@
         </is>
       </c>
       <c r="I8" s="7" t="n">
-        <v>300</v>
+        <v>900</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>37800</v>
+        <v>125000</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>126000</v>
+        <v>138889</v>
       </c>
       <c r="L8" s="7" t="n"/>
       <c r="M8" s="7">
@@ -1059,12 +1061,12 @@
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>中：交易页价格有效期为当天，但尚未固定配送门店且原价未展示</t>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
         </is>
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://www.bachhoaxanh.com/thit-heo/thit-nac-heo-300g</t>
+          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -1086,12 +1088,12 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -1101,7 +1103,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Meatcool 360-440g</t>
+          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1110,17 +1112,15 @@
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>90400</v>
+        <v>38000</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>226000</v>
-      </c>
-      <c r="L9" s="7" t="n">
-        <v>192100</v>
-      </c>
+        <v>190000</v>
+      </c>
+      <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
         <f>IF(L9&lt;&gt;"",L9,K9)</f>
         <v/>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-meatcool-400g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
@@ -1154,22 +1154,22 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>BAF</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>BAF</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo BAF khay 300g</t>
+          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -1178,13 +1178,13 @@
         </is>
       </c>
       <c r="I10" s="7" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>74000</v>
+        <v>79000</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>246667</v>
+        <v>197500</v>
       </c>
       <c r="L10" s="7" t="n"/>
       <c r="M10" s="7">
@@ -1198,7 +1198,7 @@
       </c>
       <c r="O10" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
         </is>
       </c>
     </row>
@@ -1220,22 +1220,22 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
+          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1244,13 +1244,13 @@
         </is>
       </c>
       <c r="I11" s="7" t="n">
-        <v>900</v>
+        <v>200</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>125000</v>
+        <v>33000</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>138889</v>
+        <v>165000</v>
       </c>
       <c r="L11" s="7" t="n"/>
       <c r="M11" s="7">
@@ -1264,44 +1264,44 @@
       </c>
       <c r="O11" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>小排</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Thịt đùi Meatcool túi 900g</t>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1310,13 +1310,13 @@
         </is>
       </c>
       <c r="I12" s="7" t="n">
-        <v>900</v>
+        <v>431</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>125000</v>
+        <v>124085</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>138889</v>
+        <v>287900</v>
       </c>
       <c r="L12" s="7" t="n"/>
       <c r="M12" s="7">
@@ -1325,49 +1325,49 @@
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O12" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -1376,13 +1376,13 @@
         </is>
       </c>
       <c r="I13" s="7" t="n">
-        <v>200</v>
+        <v>385</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>38000</v>
+        <v>76962</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>190000</v>
+        <v>199900</v>
       </c>
       <c r="L13" s="7" t="n"/>
       <c r="M13" s="7">
@@ -1391,144 +1391,12 @@
       </c>
       <c r="N13" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O13" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>南部</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Kingfoodmart</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Vĩnh Tân</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>Vĩnh Tân</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>猪排</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I14" s="7" t="n">
-        <v>400</v>
-      </c>
-      <c r="J14" s="7" t="n">
-        <v>79000</v>
-      </c>
-      <c r="K14" s="7" t="n">
-        <v>197500</v>
-      </c>
-      <c r="L14" s="7" t="n"/>
-      <c r="M14" s="7">
-        <f>IF(L14&lt;&gt;"",L14,K14)</f>
-        <v/>
-      </c>
-      <c r="N14" s="5" t="inlineStr">
-        <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
-        </is>
-      </c>
-      <c r="O14" s="8" t="inlineStr">
-        <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>南部</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Kingfoodmart</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Vĩnh Tân</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>Vĩnh Tân</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>后腿肉</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I15" s="7" t="n">
-        <v>200</v>
-      </c>
-      <c r="J15" s="7" t="n">
-        <v>33000</v>
-      </c>
-      <c r="K15" s="7" t="n">
-        <v>165000</v>
-      </c>
-      <c r="L15" s="7" t="n"/>
-      <c r="M15" s="7">
-        <f>IF(L15&lt;&gt;"",L15,K15)</f>
-        <v/>
-      </c>
-      <c r="N15" s="5" t="inlineStr">
-        <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
-        </is>
-      </c>
-      <c r="O15" s="8" t="inlineStr">
-        <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
+          <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
       </c>
     </row>
@@ -1537,7 +1405,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M15">
+  <conditionalFormatting sqref="M5:M13">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1555,8 +1423,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1568,7 +1434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1586,7 +1452,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>2026年7月同口径月度变化</t>
+          <t>2026年8月同口径月度变化</t>
         </is>
       </c>
     </row>
@@ -1671,7 +1537,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1694,12 +1560,12 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Bách Hóa Xanh</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>C.P.</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -1709,20 +1575,20 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Bách Hóa Xanh默认门店（待固定城市）</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>159000</v>
+        <v>199900</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>158100</v>
+        <v>199900</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>159000</v>
+        <v>199900</v>
       </c>
       <c r="I6" s="9">
         <f>IF(E6&lt;2,"",G6/F6-1)</f>
@@ -1736,35 +1602,35 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Bách Hóa Xanh</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>C.P.</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>去肋五花肉</t>
+          <t>小排</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Bách Hóa Xanh默认门店（待固定城市）</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>266667</v>
+        <v>287900</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>266667</v>
+        <v>287900</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>266667</v>
+        <v>287900</v>
       </c>
       <c r="I7" s="9">
         <f>IF(E7&lt;2,"",G7/F7-1)</f>
@@ -1778,12 +1644,12 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Bách Hóa Xanh</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>C.P.</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -1793,20 +1659,20 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Bách Hóa Xanh默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>109000</v>
+        <v>138889</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>115700</v>
+        <v>138889</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>115700</v>
+        <v>138889</v>
       </c>
       <c r="I8" s="9">
         <f>IF(E8&lt;2,"",G8/F8-1)</f>
@@ -1820,35 +1686,35 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Bách Hóa Xanh</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>C.P.</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>猪瘦肉</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Bách Hóa Xanh默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>132000</v>
+        <v>192100</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>126000</v>
+        <v>192100</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>132000</v>
+        <v>192100</v>
       </c>
       <c r="I9" s="9">
         <f>IF(E9&lt;2,"",G9/F9-1)</f>
@@ -1862,35 +1728,35 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>WinMart</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>MEATDeli</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>五花肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>WinMart默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="E10" s="7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>199900</v>
+        <v>138889</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>199900</v>
+        <v>138889</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>199900</v>
+        <v>138889</v>
       </c>
       <c r="I10" s="9">
         <f>IF(E10&lt;2,"",G10/F10-1)</f>
@@ -1904,35 +1770,35 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>WinMart</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>MEATDeli</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>小排</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>WinMart默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>287900</v>
+        <v>165000</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>287900</v>
+        <v>165000</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>287900</v>
+        <v>165000</v>
       </c>
       <c r="I11" s="9">
         <f>IF(E11&lt;2,"",G11/F11-1)</f>
@@ -1946,12 +1812,12 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>WinMart</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>MEATDeli</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -1961,20 +1827,20 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>WinMart默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>204900</v>
+        <v>190000</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>204900</v>
+        <v>190000</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>204900</v>
+        <v>190000</v>
       </c>
       <c r="I12" s="9">
         <f>IF(E12&lt;2,"",G12/F12-1)</f>
@@ -1988,35 +1854,35 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>WinMart</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>MEATDeli</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>肩肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>WinMart默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="E13" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>168900</v>
+        <v>197500</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>168900</v>
+        <v>197500</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>168900</v>
+        <v>197500</v>
       </c>
       <c r="I13" s="9">
         <f>IF(E13&lt;2,"",G13/F13-1)</f>
@@ -2024,258 +1890,6 @@
       </c>
       <c r="J13" s="5">
         <f>IF(E13&lt;2,"积累中",IF(I13&gt;=0.01,"上涨",IF(I13&lt;=-0.01,"下降","平稳")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Kingfoodmart</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Meatcool</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>后腿肉</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="F14" s="7" t="n">
-        <v>138889</v>
-      </c>
-      <c r="G14" s="7" t="n">
-        <v>138889</v>
-      </c>
-      <c r="H14" s="7" t="n">
-        <v>138889</v>
-      </c>
-      <c r="I14" s="9">
-        <f>IF(E14&lt;2,"",G14/F14-1)</f>
-        <v/>
-      </c>
-      <c r="J14" s="5">
-        <f>IF(E14&lt;2,"积累中",IF(I14&gt;=0.01,"上涨",IF(I14&lt;=-0.01,"下降","平稳")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Kingfoodmart</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Meatcool</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>梅花肉</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="n">
-        <v>11</v>
-      </c>
-      <c r="F15" s="7" t="n">
-        <v>226000</v>
-      </c>
-      <c r="G15" s="7" t="n">
-        <v>192100</v>
-      </c>
-      <c r="H15" s="7" t="n">
-        <v>192100</v>
-      </c>
-      <c r="I15" s="9">
-        <f>IF(E15&lt;2,"",G15/F15-1)</f>
-        <v/>
-      </c>
-      <c r="J15" s="5">
-        <f>IF(E15&lt;2,"积累中",IF(I15&gt;=0.01,"上涨",IF(I15&lt;=-0.01,"下降","平稳")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Kingfoodmart</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Meatcool</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>猪排</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
-        </is>
-      </c>
-      <c r="E16" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="F16" s="7" t="n">
-        <v>138889</v>
-      </c>
-      <c r="G16" s="7" t="n">
-        <v>138889</v>
-      </c>
-      <c r="H16" s="7" t="n">
-        <v>138889</v>
-      </c>
-      <c r="I16" s="9">
-        <f>IF(E16&lt;2,"",G16/F16-1)</f>
-        <v/>
-      </c>
-      <c r="J16" s="5">
-        <f>IF(E16&lt;2,"积累中",IF(I16&gt;=0.01,"上涨",IF(I16&lt;=-0.01,"下降","平稳")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>Kingfoodmart</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Vĩnh Tân</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>后腿肉</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="F17" s="7" t="n">
-        <v>165000</v>
-      </c>
-      <c r="G17" s="7" t="n">
-        <v>165000</v>
-      </c>
-      <c r="H17" s="7" t="n">
-        <v>165000</v>
-      </c>
-      <c r="I17" s="9">
-        <f>IF(E17&lt;2,"",G17/F17-1)</f>
-        <v/>
-      </c>
-      <c r="J17" s="5">
-        <f>IF(E17&lt;2,"积累中",IF(I17&gt;=0.01,"上涨",IF(I17&lt;=-0.01,"下降","平稳")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Kingfoodmart</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Vĩnh Tân</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>梅花肉</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="F18" s="7" t="n">
-        <v>185000</v>
-      </c>
-      <c r="G18" s="7" t="n">
-        <v>190000</v>
-      </c>
-      <c r="H18" s="7" t="n">
-        <v>190000</v>
-      </c>
-      <c r="I18" s="9">
-        <f>IF(E18&lt;2,"",G18/F18-1)</f>
-        <v/>
-      </c>
-      <c r="J18" s="5">
-        <f>IF(E18&lt;2,"积累中",IF(I18&gt;=0.01,"上涨",IF(I18&lt;=-0.01,"下降","平稳")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>Kingfoodmart</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Vĩnh Tân</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>猪排</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="n">
-        <v>11</v>
-      </c>
-      <c r="F19" s="7" t="n">
-        <v>197500</v>
-      </c>
-      <c r="G19" s="7" t="n">
-        <v>197500</v>
-      </c>
-      <c r="H19" s="7" t="n">
-        <v>197500</v>
-      </c>
-      <c r="I19" s="9">
-        <f>IF(E19&lt;2,"",G19/F19-1)</f>
-        <v/>
-      </c>
-      <c r="J19" s="5">
-        <f>IF(E19&lt;2,"积累中",IF(I19&gt;=0.01,"上涨",IF(I19&lt;=-0.01,"下降","平稳")))</f>
         <v/>
       </c>
     </row>
@@ -2284,7 +1898,7 @@
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="I5:I19">
+  <conditionalFormatting sqref="I5:I13">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="1">
       <formula>0.01</formula>
     </cfRule>
@@ -2362,12 +1976,12 @@
     <row r="5" ht="58" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Bách Hóa Xanh</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>C.P. Vietnam / C.P.</t>
+          <t>GREENFEED / Meatcool</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -2382,12 +1996,12 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>中：交易页价格有效期为当天，但尚未固定配送门店且原价未展示</t>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>https://www.bachhoaxanh.com/thit-heo/ba-roi-heo</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-meatcool-400g</t>
         </is>
       </c>
     </row>
@@ -2399,7 +2013,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED / Meatcool</t>
+          <t>BAF / BAF</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -2419,7 +2033,7 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-meatcool-400g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
         </is>
       </c>
     </row>
@@ -2431,7 +2045,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>BAF / BAF</t>
+          <t>Vĩnh Tân / Vĩnh Tân</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -2451,24 +2065,24 @@
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
     <row r="8" ht="58" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân / Vĩnh Tân</t>
+          <t>Masan / MEATDeli</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>A-零售交易页</t>
+          <t>A-官方交易页</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -2478,12 +2092,12 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-01
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-01</t>
+          <t>越南猪肉零售价格日报｜2026-08-02</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 05:42。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 05:41。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,12 +588,12 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>9条在售商品</t>
+          <t>6条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>渠道：Kingfoodmart、WinMart</t>
+          <t>渠道：Kingfoodmart</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -610,12 +610,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>4个</t>
+          <t>3个</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>BAF、MEATDeli、Meatcool、Vĩnh Tân</t>
+          <t>BAF、Meatcool、Vĩnh Tân</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -632,7 +632,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>0组</t>
+          <t>6组</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-01</t>
+          <t>越南猪肉零售明细｜2026-08-02</t>
         </is>
       </c>
     </row>
@@ -1199,204 +1199,6 @@
       <c r="O10" s="8" t="inlineStr">
         <is>
           <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>南部</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Kingfoodmart</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Vĩnh Tân</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>Vĩnh Tân</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>后腿肉</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I11" s="7" t="n">
-        <v>200</v>
-      </c>
-      <c r="J11" s="7" t="n">
-        <v>33000</v>
-      </c>
-      <c r="K11" s="7" t="n">
-        <v>165000</v>
-      </c>
-      <c r="L11" s="7" t="n"/>
-      <c r="M11" s="7">
-        <f>IF(L11&lt;&gt;"",L11,K11)</f>
-        <v/>
-      </c>
-      <c r="N11" s="5" t="inlineStr">
-        <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
-        </is>
-      </c>
-      <c r="O11" s="8" t="inlineStr">
-        <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>小排</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I12" s="7" t="n">
-        <v>431</v>
-      </c>
-      <c r="J12" s="7" t="n">
-        <v>124085</v>
-      </c>
-      <c r="K12" s="7" t="n">
-        <v>287900</v>
-      </c>
-      <c r="L12" s="7" t="n"/>
-      <c r="M12" s="7">
-        <f>IF(L12&lt;&gt;"",L12,K12)</f>
-        <v/>
-      </c>
-      <c r="N12" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O12" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>五花肉</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I13" s="7" t="n">
-        <v>385</v>
-      </c>
-      <c r="J13" s="7" t="n">
-        <v>76962</v>
-      </c>
-      <c r="K13" s="7" t="n">
-        <v>199900</v>
-      </c>
-      <c r="L13" s="7" t="n"/>
-      <c r="M13" s="7">
-        <f>IF(L13&lt;&gt;"",L13,K13)</f>
-        <v/>
-      </c>
-      <c r="N13" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O13" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1207,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M13">
+  <conditionalFormatting sqref="M5:M10">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1420,9 +1222,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1537,7 +1336,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1663,7 +1462,7 @@
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>138889</v>
@@ -1705,7 +1504,7 @@
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>192100</v>
@@ -1747,7 +1546,7 @@
         </is>
       </c>
       <c r="E10" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" s="7" t="n">
         <v>138889</v>
@@ -1831,7 +1630,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>190000</v>
@@ -1873,7 +1672,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>197500</v>
@@ -1916,7 +1715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2069,38 +1868,6 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="58" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Masan / MEATDeli</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>A-官方交易页</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>实际价/kg = 促销价/kg（如有），否则常规价/kg；包装价÷重量(kg)用于交叉核验。</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
@@ -2110,7 +1877,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-02
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-02</t>
+          <t>越南猪肉零售价格日报｜2026-08-03</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 05:41。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 05:39。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>渠道：Kingfoodmart</t>
+          <t>渠道：Kingfoodmart、WinMart</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -610,12 +610,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>3个</t>
+          <t>4个</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>BAF、Meatcool、Vĩnh Tân</t>
+          <t>BAF、MEATDeli、Meatcool、Vĩnh Tân</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -632,7 +632,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>6组</t>
+          <t>8组</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-02</t>
+          <t>越南猪肉零售明细｜2026-08-03</t>
         </is>
       </c>
     </row>
@@ -956,22 +956,22 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
+          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -980,13 +980,13 @@
         </is>
       </c>
       <c r="I7" s="7" t="n">
-        <v>900</v>
+        <v>200</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>125000</v>
+        <v>38000</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>138889</v>
+        <v>190000</v>
       </c>
       <c r="L7" s="7" t="n"/>
       <c r="M7" s="7">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
@@ -1022,22 +1022,22 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Thịt đùi Meatcool túi 900g</t>
+          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1046,13 +1046,13 @@
         </is>
       </c>
       <c r="I8" s="7" t="n">
-        <v>900</v>
+        <v>400</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>125000</v>
+        <v>79000</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>138889</v>
+        <v>197500</v>
       </c>
       <c r="L8" s="7" t="n"/>
       <c r="M8" s="7">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
         </is>
       </c>
     </row>
@@ -1098,12 +1098,12 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
+          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1115,10 +1115,10 @@
         <v>200</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>38000</v>
+        <v>33000</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>190000</v>
+        <v>165000</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
@@ -1132,44 +1132,44 @@
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>小排</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -1178,13 +1178,13 @@
         </is>
       </c>
       <c r="I10" s="7" t="n">
-        <v>400</v>
+        <v>431</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>79000</v>
+        <v>124085</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>197500</v>
+        <v>287900</v>
       </c>
       <c r="L10" s="7" t="n"/>
       <c r="M10" s="7">
@@ -1193,12 +1193,12 @@
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O10" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>
@@ -1336,7 +1336,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1420,7 +1420,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1504,7 +1504,7 @@
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>192100</v>
@@ -1588,7 +1588,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>165000</v>
@@ -1630,7 +1630,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>190000</v>
@@ -1672,7 +1672,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>197500</v>
@@ -1715,7 +1715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1868,6 +1868,38 @@
         </is>
       </c>
     </row>
+    <row r="8" ht="58" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>WinMart</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Masan / MEATDeli</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>A-官方交易页</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>实际价/kg = 促销价/kg（如有），否则常规价/kg；包装价÷重量(kg)用于交叉核验。</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>中：官方交易页，但尚未固定配送门店</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
@@ -1877,6 +1909,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-03
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-03</t>
+          <t>越南猪肉零售价格日报｜2026-08-04</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 05:39。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 05:41。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>6条在售商品</t>
+          <t>8条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-03</t>
+          <t>越南猪肉零售明细｜2026-08-04</t>
         </is>
       </c>
     </row>
@@ -956,22 +956,22 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
+          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -980,13 +980,13 @@
         </is>
       </c>
       <c r="I7" s="7" t="n">
-        <v>200</v>
+        <v>900</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>38000</v>
+        <v>125000</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>190000</v>
+        <v>138889</v>
       </c>
       <c r="L7" s="7" t="n"/>
       <c r="M7" s="7">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
+          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -1022,22 +1022,22 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
+          <t>Thịt đùi Meatcool túi 900g</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1046,13 +1046,13 @@
         </is>
       </c>
       <c r="I8" s="7" t="n">
-        <v>400</v>
+        <v>900</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>79000</v>
+        <v>125000</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>197500</v>
+        <v>138889</v>
       </c>
       <c r="L8" s="7" t="n"/>
       <c r="M8" s="7">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -1098,12 +1098,12 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
+          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1115,10 +1115,10 @@
         <v>200</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>33000</v>
+        <v>38000</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>165000</v>
+        <v>190000</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
@@ -1132,44 +1132,44 @@
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>全国渠道</t>
+          <t>南部</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>WinMart默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>WinMart</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Masan</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>MEATDeli</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>小排</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
+          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -1178,13 +1178,13 @@
         </is>
       </c>
       <c r="I10" s="7" t="n">
-        <v>431</v>
+        <v>400</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>124085</v>
+        <v>79000</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>287900</v>
+        <v>197500</v>
       </c>
       <c r="L10" s="7" t="n"/>
       <c r="M10" s="7">
@@ -1193,10 +1193,142 @@
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+        </is>
+      </c>
+      <c r="O10" s="8" t="inlineStr">
+        <is>
+          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>南部</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>胡志明市/Kingfoodmart默认门店</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Kingfoodmart</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Vĩnh Tân</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Vĩnh Tân</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>后腿肉</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>冷鲜</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>33000</v>
+      </c>
+      <c r="K11" s="7" t="n">
+        <v>165000</v>
+      </c>
+      <c r="L11" s="7" t="n"/>
+      <c r="M11" s="7">
+        <f>IF(L11&lt;&gt;"",L11,K11)</f>
+        <v/>
+      </c>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+        </is>
+      </c>
+      <c r="O11" s="8" t="inlineStr">
+        <is>
+          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>全国渠道</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>WinMart默认门店（待固定城市）</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>WinMart</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Masan</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>MEATDeli</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>小排</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>冷鲜</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="n">
+        <v>431</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>124085</v>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>287900</v>
+      </c>
+      <c r="L12" s="7" t="n"/>
+      <c r="M12" s="7">
+        <f>IF(L12&lt;&gt;"",L12,K12)</f>
+        <v/>
+      </c>
+      <c r="N12" s="5" t="inlineStr">
+        <is>
           <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
-      <c r="O10" s="8" t="inlineStr">
+      <c r="O12" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
@@ -1207,7 +1339,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M10">
+  <conditionalFormatting sqref="M5:M12">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1222,6 +1354,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1336,7 +1470,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1420,7 +1554,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1462,7 +1596,7 @@
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>138889</v>
@@ -1504,7 +1638,7 @@
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>192100</v>
@@ -1546,7 +1680,7 @@
         </is>
       </c>
       <c r="E10" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F10" s="7" t="n">
         <v>138889</v>
@@ -1588,7 +1722,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>165000</v>
@@ -1630,7 +1764,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>190000</v>
@@ -1672,7 +1806,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>197500</v>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-04
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-04</t>
+          <t>越南猪肉零售价格日报｜2026-08-05</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 05:41。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 05:45。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-04</t>
+          <t>越南猪肉零售明细｜2026-08-05</t>
         </is>
       </c>
     </row>
@@ -890,22 +890,22 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>BAF</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>BAF</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo BAF khay 300g</t>
+          <t>Ba rọi heo Meatcool 360-440g</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -914,15 +914,17 @@
         </is>
       </c>
       <c r="I6" s="7" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>74000</v>
+        <v>99600</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>246667</v>
-      </c>
-      <c r="L6" s="7" t="n"/>
+        <v>249000</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <v>195000</v>
+      </c>
       <c r="M6" s="7">
         <f>IF(L6&lt;&gt;"",L6,K6)</f>
         <v/>
@@ -934,7 +936,7 @@
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/sap-mo-ban-ba-roi-heo-meatcool-400g-ol312263</t>
         </is>
       </c>
     </row>
@@ -956,22 +958,22 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>BAF</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>BAF</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
+          <t>Nạc dăm heo BAF khay 300g</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -980,13 +982,13 @@
         </is>
       </c>
       <c r="I7" s="7" t="n">
-        <v>900</v>
+        <v>300</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>125000</v>
+        <v>74000</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>138889</v>
+        <v>246667</v>
       </c>
       <c r="L7" s="7" t="n"/>
       <c r="M7" s="7">
@@ -1000,7 +1002,7 @@
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
         </is>
       </c>
     </row>
@@ -1088,22 +1090,22 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
+          <t>Cốt lết heo Meatcool khay 300g</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1112,13 +1114,13 @@
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>38000</v>
+        <v>35000</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>190000</v>
+        <v>116667</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
@@ -1132,7 +1134,7 @@
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
+          <t>https://kingfoodmart.com/thit-heo/sap-mo-ban-cot-let-heo-meatcool-khay-300g-ol344147</t>
         </is>
       </c>
     </row>
@@ -1164,12 +1166,12 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
+          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -1178,13 +1180,13 @@
         </is>
       </c>
       <c r="I10" s="7" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>79000</v>
+        <v>38000</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>197500</v>
+        <v>190000</v>
       </c>
       <c r="L10" s="7" t="n"/>
       <c r="M10" s="7">
@@ -1198,7 +1200,7 @@
       </c>
       <c r="O10" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
@@ -1230,12 +1232,12 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
+          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1244,13 +1246,13 @@
         </is>
       </c>
       <c r="I11" s="7" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>33000</v>
+        <v>79000</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>165000</v>
+        <v>197500</v>
       </c>
       <c r="L11" s="7" t="n"/>
       <c r="M11" s="7">
@@ -1264,7 +1266,7 @@
       </c>
       <c r="O11" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
         </is>
       </c>
     </row>
@@ -1367,7 +1369,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1470,7 +1472,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1554,7 +1556,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1587,7 +1589,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -1596,16 +1598,16 @@
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>138889</v>
+        <v>195000</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>138889</v>
+        <v>195000</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>138889</v>
+        <v>195000</v>
       </c>
       <c r="I8" s="9">
         <f>IF(E8&lt;2,"",G8/F8-1)</f>
@@ -1629,7 +1631,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -1641,13 +1643,13 @@
         <v>4</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>192100</v>
+        <v>138889</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>192100</v>
+        <v>138889</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>192100</v>
+        <v>138889</v>
       </c>
       <c r="I9" s="9">
         <f>IF(E9&lt;2,"",G9/F9-1)</f>
@@ -1671,7 +1673,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -1680,16 +1682,16 @@
         </is>
       </c>
       <c r="E10" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>138889</v>
+        <v>192100</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>138889</v>
+        <v>192100</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>138889</v>
+        <v>192100</v>
       </c>
       <c r="I10" s="9">
         <f>IF(E10&lt;2,"",G10/F10-1)</f>
@@ -1708,12 +1710,12 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -1722,16 +1724,16 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>165000</v>
+        <v>138889</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>165000</v>
+        <v>116667</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>165000</v>
+        <v>138889</v>
       </c>
       <c r="I11" s="9">
         <f>IF(E11&lt;2,"",G11/F11-1)</f>
@@ -1755,7 +1757,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -1764,16 +1766,16 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>190000</v>
+        <v>165000</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>190000</v>
+        <v>165000</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>190000</v>
+        <v>165000</v>
       </c>
       <c r="I12" s="9">
         <f>IF(E12&lt;2,"",G12/F12-1)</f>
@@ -1797,7 +1799,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -1806,16 +1808,16 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>197500</v>
+        <v>190000</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>197500</v>
+        <v>190000</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>197500</v>
+        <v>190000</v>
       </c>
       <c r="I13" s="9">
         <f>IF(E13&lt;2,"",G13/F13-1)</f>
@@ -1823,6 +1825,48 @@
       </c>
       <c r="J13" s="5">
         <f>IF(E13&lt;2,"积累中",IF(I13&gt;=0.01,"上涨",IF(I13&lt;=-0.01,"下降","平稳")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Kingfoodmart</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Vĩnh Tân</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>猪排</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>胡志明市/Kingfoodmart默认门店</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>197500</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>197500</v>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>197500</v>
+      </c>
+      <c r="I14" s="9">
+        <f>IF(E14&lt;2,"",G14/F14-1)</f>
+        <v/>
+      </c>
+      <c r="J14" s="5">
+        <f>IF(E14&lt;2,"积累中",IF(I14&gt;=0.01,"上涨",IF(I14&lt;=-0.01,"下降","平稳")))</f>
         <v/>
       </c>
     </row>
@@ -1831,7 +1875,7 @@
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="I5:I13">
+  <conditionalFormatting sqref="I5:I14">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="1">
       <formula>0.01</formula>
     </cfRule>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-05
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-05</t>
+          <t>越南猪肉零售价格日报｜2026-08-06</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 05:45。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 05:42。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>8条在售商品</t>
+          <t>9条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -632,7 +632,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>8组</t>
+          <t>10组</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O12"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-05</t>
+          <t>越南猪肉零售明细｜2026-08-06</t>
         </is>
       </c>
     </row>
@@ -936,7 +936,7 @@
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/sap-mo-ban-ba-roi-heo-meatcool-400g-ol312263</t>
+          <t>https://kingfoodmart.com/thit-heo/ba-roi-heo-meatcool-400g</t>
         </is>
       </c>
     </row>
@@ -1134,7 +1134,7 @@
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/sap-mo-ban-cot-let-heo-meatcool-khay-300g-ol344147</t>
+          <t>https://kingfoodmart.com/thit-heo/cot-let-heo-meatcool-khay-300g</t>
         </is>
       </c>
     </row>
@@ -1333,6 +1333,72 @@
       <c r="O12" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>全国渠道</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>WinMart默认门店（待固定城市）</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>WinMart</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Masan</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>MEATDeli</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>五花肉</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>冷鲜</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>385</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>76962</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>199900</v>
+      </c>
+      <c r="L13" s="7" t="n"/>
+      <c r="M13" s="7">
+        <f>IF(L13&lt;&gt;"",L13,K13)</f>
+        <v/>
+      </c>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>中：官方交易页，但尚未固定配送门店</t>
+        </is>
+      </c>
+      <c r="O13" s="8" t="inlineStr">
+        <is>
+          <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1407,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M12">
+  <conditionalFormatting sqref="M5:M13">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1358,6 +1424,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1472,7 +1539,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1514,7 +1581,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1556,7 +1623,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1598,7 +1665,7 @@
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>195000</v>
@@ -1640,7 +1707,7 @@
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>138889</v>
@@ -1682,7 +1749,7 @@
         </is>
       </c>
       <c r="E10" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F10" s="7" t="n">
         <v>192100</v>
@@ -1724,7 +1791,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1808,7 +1875,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>190000</v>
@@ -1850,7 +1917,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>197500</v>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-07
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-06</t>
+          <t>越南猪肉零售价格日报｜2026-08-07</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 05:42。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 08:04。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>9条在售商品</t>
+          <t>10条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-06</t>
+          <t>越南猪肉零售明细｜2026-08-07</t>
         </is>
       </c>
     </row>
@@ -1364,12 +1364,12 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>五花肉</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
+          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -1378,13 +1378,13 @@
         </is>
       </c>
       <c r="I13" s="7" t="n">
-        <v>385</v>
+        <v>400</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>76962</v>
+        <v>81960</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>199900</v>
+        <v>204900</v>
       </c>
       <c r="L13" s="7" t="n"/>
       <c r="M13" s="7">
@@ -1397,6 +1397,72 @@
         </is>
       </c>
       <c r="O13" s="8" t="inlineStr">
+        <is>
+          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>全国渠道</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>WinMart默认门店（待固定城市）</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>WinMart</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Masan</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>MEATDeli</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>五花肉</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>冷鲜</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>385</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>76962</v>
+      </c>
+      <c r="K14" s="7" t="n">
+        <v>199900</v>
+      </c>
+      <c r="L14" s="7" t="n"/>
+      <c r="M14" s="7">
+        <f>IF(L14&lt;&gt;"",L14,K14)</f>
+        <v/>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>中：官方交易页，但尚未固定配送门店</t>
+        </is>
+      </c>
+      <c r="O14" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
@@ -1407,7 +1473,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M13">
+  <conditionalFormatting sqref="M5:M14">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1425,6 +1491,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1436,7 +1503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1539,7 +1606,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1581,7 +1648,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1623,7 +1690,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1646,35 +1713,35 @@
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>五花肉</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>195000</v>
+        <v>204900</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>195000</v>
+        <v>204900</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>195000</v>
+        <v>204900</v>
       </c>
       <c r="I8" s="9">
         <f>IF(E8&lt;2,"",G8/F8-1)</f>
@@ -1698,7 +1765,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -1707,16 +1774,16 @@
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>138889</v>
+        <v>195000</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>138889</v>
+        <v>195000</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>138889</v>
+        <v>195000</v>
       </c>
       <c r="I9" s="9">
         <f>IF(E9&lt;2,"",G9/F9-1)</f>
@@ -1740,7 +1807,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -1752,13 +1819,13 @@
         <v>6</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>192100</v>
+        <v>138889</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>192100</v>
+        <v>138889</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>192100</v>
+        <v>138889</v>
       </c>
       <c r="I10" s="9">
         <f>IF(E10&lt;2,"",G10/F10-1)</f>
@@ -1782,7 +1849,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -1791,16 +1858,16 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>138889</v>
+        <v>192100</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>116667</v>
+        <v>192100</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>138889</v>
+        <v>192100</v>
       </c>
       <c r="I11" s="9">
         <f>IF(E11&lt;2,"",G11/F11-1)</f>
@@ -1819,12 +1886,12 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -1833,16 +1900,16 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>165000</v>
+        <v>138889</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>165000</v>
+        <v>116667</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>165000</v>
+        <v>127778</v>
       </c>
       <c r="I12" s="9">
         <f>IF(E12&lt;2,"",G12/F12-1)</f>
@@ -1866,7 +1933,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -1875,16 +1942,16 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>190000</v>
+        <v>165000</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>190000</v>
+        <v>165000</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>190000</v>
+        <v>165000</v>
       </c>
       <c r="I13" s="9">
         <f>IF(E13&lt;2,"",G13/F13-1)</f>
@@ -1908,7 +1975,7 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -1917,16 +1984,16 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>197500</v>
+        <v>190000</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>197500</v>
+        <v>190000</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>197500</v>
+        <v>190000</v>
       </c>
       <c r="I14" s="9">
         <f>IF(E14&lt;2,"",G14/F14-1)</f>
@@ -1934,6 +2001,48 @@
       </c>
       <c r="J14" s="5">
         <f>IF(E14&lt;2,"积累中",IF(I14&gt;=0.01,"上涨",IF(I14&lt;=-0.01,"下降","平稳")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Kingfoodmart</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Vĩnh Tân</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>猪排</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>胡志明市/Kingfoodmart默认门店</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>197500</v>
+      </c>
+      <c r="G15" s="7" t="n">
+        <v>197500</v>
+      </c>
+      <c r="H15" s="7" t="n">
+        <v>197500</v>
+      </c>
+      <c r="I15" s="9">
+        <f>IF(E15&lt;2,"",G15/F15-1)</f>
+        <v/>
+      </c>
+      <c r="J15" s="5">
+        <f>IF(E15&lt;2,"积累中",IF(I15&gt;=0.01,"上涨",IF(I15&lt;=-0.01,"下降","平稳")))</f>
         <v/>
       </c>
     </row>
@@ -1942,7 +2051,7 @@
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="I5:I14">
+  <conditionalFormatting sqref="I5:I15">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="1">
       <formula>0.01</formula>
     </cfRule>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-08
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-08</t>
+          <t>越南猪肉零售价格日报｜2026-08-09</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 05:18。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 05:02。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>10条在售商品</t>
+          <t>9条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-08</t>
+          <t>越南猪肉零售明细｜2026-08-09</t>
         </is>
       </c>
     </row>
@@ -837,7 +837,7 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo đầu giòn Meatcool Premium 360-440g</t>
+          <t>Nạc dăm heo Meatcool 360-440g</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -849,13 +849,13 @@
         <v>400</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>130800</v>
+        <v>90400</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>327000</v>
+        <v>226000</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>277950</v>
+        <v>192100</v>
       </c>
       <c r="M5" s="7">
         <f>IF(L5&lt;&gt;"",L5,K5)</f>
@@ -868,7 +868,7 @@
       </c>
       <c r="O5" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-dau-gion-meatcool-premium-400g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-meatcool-400g</t>
         </is>
       </c>
     </row>
@@ -890,22 +890,22 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>BAF</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>BAF</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>五花肉</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Ba rọi heo Meatcool 360-440g</t>
+          <t>Nạc dăm heo BAF khay 300g</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -914,17 +914,15 @@
         </is>
       </c>
       <c r="I6" s="7" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>99600</v>
+        <v>74000</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>249000</v>
-      </c>
-      <c r="L6" s="7" t="n">
-        <v>195000</v>
-      </c>
+        <v>246667</v>
+      </c>
+      <c r="L6" s="7" t="n"/>
       <c r="M6" s="7">
         <f>IF(L6&lt;&gt;"",L6,K6)</f>
         <v/>
@@ -936,7 +934,7 @@
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/ba-roi-heo-meatcool-400g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
         </is>
       </c>
     </row>
@@ -958,22 +956,22 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>BAF</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>BAF</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo BAF khay 300g</t>
+          <t>Thịt đùi Meatcool túi 900g</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -982,13 +980,13 @@
         </is>
       </c>
       <c r="I7" s="7" t="n">
-        <v>300</v>
+        <v>900</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>74000</v>
+        <v>125000</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>246667</v>
+        <v>138889</v>
       </c>
       <c r="L7" s="7" t="n"/>
       <c r="M7" s="7">
@@ -1002,7 +1000,7 @@
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -1034,12 +1032,12 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Thịt đùi Meatcool túi 900g</t>
+          <t>Cốt lết heo Meatcool khay 300g</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1048,13 +1046,13 @@
         </is>
       </c>
       <c r="I8" s="7" t="n">
-        <v>900</v>
+        <v>300</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>125000</v>
+        <v>35000</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>138889</v>
+        <v>116667</v>
       </c>
       <c r="L8" s="7" t="n"/>
       <c r="M8" s="7">
@@ -1068,7 +1066,7 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/cot-let-heo-meatcool-khay-300g</t>
         </is>
       </c>
     </row>
@@ -1090,22 +1088,22 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Cốt lết heo Meatcool khay 300g</t>
+          <t>Nạc dăm heo Vĩnh Tân 400g</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1114,13 +1112,13 @@
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>35000</v>
+        <v>77000</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>116667</v>
+        <v>192500</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
@@ -1134,7 +1132,7 @@
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/cot-let-heo-meatcool-khay-300g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-400g-1-khay-63124</t>
         </is>
       </c>
     </row>
@@ -1166,12 +1164,12 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Vĩnh Tân 400g</t>
+          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -1183,10 +1181,10 @@
         <v>400</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>77000</v>
+        <v>79000</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>192500</v>
+        <v>197500</v>
       </c>
       <c r="L10" s="7" t="n"/>
       <c r="M10" s="7">
@@ -1200,7 +1198,7 @@
       </c>
       <c r="O10" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-400g-1-khay-63124</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
         </is>
       </c>
     </row>
@@ -1232,12 +1230,12 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
+          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1246,13 +1244,13 @@
         </is>
       </c>
       <c r="I11" s="7" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>79000</v>
+        <v>33000</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>197500</v>
+        <v>165000</v>
       </c>
       <c r="L11" s="7" t="n"/>
       <c r="M11" s="7">
@@ -1266,44 +1264,44 @@
       </c>
       <c r="O11" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>小排</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1312,13 +1310,13 @@
         </is>
       </c>
       <c r="I12" s="7" t="n">
-        <v>200</v>
+        <v>431</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>33000</v>
+        <v>124085</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>165000</v>
+        <v>287900</v>
       </c>
       <c r="L12" s="7" t="n"/>
       <c r="M12" s="7">
@@ -1327,12 +1325,12 @@
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O12" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>
@@ -1364,12 +1362,12 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>小排</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -1378,13 +1376,13 @@
         </is>
       </c>
       <c r="I13" s="7" t="n">
-        <v>431</v>
+        <v>385</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>124085</v>
+        <v>76962</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>287900</v>
+        <v>199900</v>
       </c>
       <c r="L13" s="7" t="n"/>
       <c r="M13" s="7">
@@ -1397,72 +1395,6 @@
         </is>
       </c>
       <c r="O13" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>五花肉</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I14" s="7" t="n">
-        <v>385</v>
-      </c>
-      <c r="J14" s="7" t="n">
-        <v>76962</v>
-      </c>
-      <c r="K14" s="7" t="n">
-        <v>199900</v>
-      </c>
-      <c r="L14" s="7" t="n"/>
-      <c r="M14" s="7">
-        <f>IF(L14&lt;&gt;"",L14,K14)</f>
-        <v/>
-      </c>
-      <c r="N14" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O14" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
@@ -1473,7 +1405,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M14">
+  <conditionalFormatting sqref="M5:M13">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1491,7 +1423,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1606,7 +1537,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1648,7 +1579,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1690,7 +1621,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1816,7 +1747,7 @@
         </is>
       </c>
       <c r="E10" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F10" s="7" t="n">
         <v>138889</v>
@@ -1858,13 +1789,13 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>192100</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>277950</v>
+        <v>192100</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>192100</v>
@@ -1900,7 +1831,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>138889</v>
@@ -1942,7 +1873,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>165000</v>
@@ -1984,7 +1915,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>190000</v>
@@ -2026,7 +1957,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>197500</v>
@@ -2154,7 +2085,7 @@
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-dau-gion-meatcool-premium-400g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-meatcool-400g</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-09
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-09</t>
+          <t>越南猪肉零售价格日报｜2026-08-10</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 05:02。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 05:04。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-09</t>
+          <t>越南猪肉零售明细｜2026-08-10</t>
         </is>
       </c>
     </row>
@@ -966,12 +966,12 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Thịt đùi Meatcool túi 900g</t>
+          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/sap-mo-ban-cot-let-meatcool-tui-900g-ol341387</t>
         </is>
       </c>
     </row>
@@ -1032,12 +1032,12 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Cốt lết heo Meatcool khay 300g</t>
+          <t>Thịt đùi Meatcool túi 900g</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1046,13 +1046,13 @@
         </is>
       </c>
       <c r="I8" s="7" t="n">
-        <v>300</v>
+        <v>900</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>35000</v>
+        <v>125000</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>116667</v>
+        <v>138889</v>
       </c>
       <c r="L8" s="7" t="n"/>
       <c r="M8" s="7">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/cot-let-heo-meatcool-khay-300g</t>
+          <t>https://kingfoodmart.com/thit-heo/sap-mo-ban-thit-dui-meatcool-tui-900g-ol341387</t>
         </is>
       </c>
     </row>
@@ -1537,7 +1537,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1579,7 +1579,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1621,7 +1621,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1747,7 +1747,7 @@
         </is>
       </c>
       <c r="E10" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F10" s="7" t="n">
         <v>138889</v>
@@ -1789,7 +1789,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>192100</v>
@@ -1831,13 +1831,13 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>138889</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>116667</v>
+        <v>138889</v>
       </c>
       <c r="H12" s="7" t="n">
         <v>116667</v>
@@ -1873,7 +1873,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>165000</v>
@@ -1915,7 +1915,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>190000</v>
@@ -1957,7 +1957,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>197500</v>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-10
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-10</t>
+          <t>越南猪肉零售价格日报｜2026-08-11</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 05:04。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 05:20。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>9条在售商品</t>
+          <t>10条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-10</t>
+          <t>越南猪肉零售明细｜2026-08-11</t>
         </is>
       </c>
     </row>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/sap-mo-ban-thit-dui-meatcool-tui-900g-ol341387</t>
+          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -1296,12 +1296,12 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>小排</t>
+          <t>肩肉</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
+          <t>MEATDELI Thịt Nạc vai heo (S)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1310,13 +1310,13 @@
         </is>
       </c>
       <c r="I12" s="7" t="n">
-        <v>431</v>
+        <v>440</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>124085</v>
+        <v>74316</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>287900</v>
+        <v>168900</v>
       </c>
       <c r="L12" s="7" t="n"/>
       <c r="M12" s="7">
@@ -1330,7 +1330,7 @@
       </c>
       <c r="O12" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
         </is>
       </c>
     </row>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>五花肉</t>
+          <t>小排</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -1376,13 +1376,13 @@
         </is>
       </c>
       <c r="I13" s="7" t="n">
-        <v>385</v>
+        <v>431</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>76962</v>
+        <v>124085</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>199900</v>
+        <v>287900</v>
       </c>
       <c r="L13" s="7" t="n"/>
       <c r="M13" s="7">
@@ -1395,6 +1395,72 @@
         </is>
       </c>
       <c r="O13" s="8" t="inlineStr">
+        <is>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>全国渠道</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>WinMart默认门店（待固定城市）</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>WinMart</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Masan</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>MEATDeli</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>五花肉</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>冷鲜</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>385</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>76962</v>
+      </c>
+      <c r="K14" s="7" t="n">
+        <v>199900</v>
+      </c>
+      <c r="L14" s="7" t="n"/>
+      <c r="M14" s="7">
+        <f>IF(L14&lt;&gt;"",L14,K14)</f>
+        <v/>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>中：官方交易页，但尚未固定配送门店</t>
+        </is>
+      </c>
+      <c r="O14" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
@@ -1405,7 +1471,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M13">
+  <conditionalFormatting sqref="M5:M14">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1423,6 +1489,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1434,7 +1501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1537,7 +1604,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1579,7 +1646,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1621,7 +1688,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1686,35 +1753,35 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>五花肉</t>
+          <t>肩肉</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>195000</v>
+        <v>168900</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>195000</v>
+        <v>168900</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>195000</v>
+        <v>168900</v>
       </c>
       <c r="I9" s="9">
         <f>IF(E9&lt;2,"",G9/F9-1)</f>
@@ -1738,7 +1805,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -1747,16 +1814,16 @@
         </is>
       </c>
       <c r="E10" s="7" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>138889</v>
+        <v>195000</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>138889</v>
+        <v>195000</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>138889</v>
+        <v>195000</v>
       </c>
       <c r="I10" s="9">
         <f>IF(E10&lt;2,"",G10/F10-1)</f>
@@ -1780,7 +1847,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -1792,13 +1859,13 @@
         <v>10</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>192100</v>
+        <v>138889</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>192100</v>
+        <v>138889</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>192100</v>
+        <v>138889</v>
       </c>
       <c r="I11" s="9">
         <f>IF(E11&lt;2,"",G11/F11-1)</f>
@@ -1822,7 +1889,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -1831,16 +1898,16 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>138889</v>
+        <v>192100</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>138889</v>
+        <v>192100</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>116667</v>
+        <v>192100</v>
       </c>
       <c r="I12" s="9">
         <f>IF(E12&lt;2,"",G12/F12-1)</f>
@@ -1859,12 +1926,12 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -1873,16 +1940,16 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>165000</v>
+        <v>138889</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>165000</v>
+        <v>138889</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>165000</v>
+        <v>127778</v>
       </c>
       <c r="I13" s="9">
         <f>IF(E13&lt;2,"",G13/F13-1)</f>
@@ -1906,7 +1973,7 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -1915,16 +1982,16 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>190000</v>
+        <v>165000</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>192500</v>
+        <v>165000</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>190000</v>
+        <v>165000</v>
       </c>
       <c r="I14" s="9">
         <f>IF(E14&lt;2,"",G14/F14-1)</f>
@@ -1948,7 +2015,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -1957,16 +2024,16 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>197500</v>
+        <v>190000</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>197500</v>
+        <v>192500</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>197500</v>
+        <v>190000</v>
       </c>
       <c r="I15" s="9">
         <f>IF(E15&lt;2,"",G15/F15-1)</f>
@@ -1974,6 +2041,48 @@
       </c>
       <c r="J15" s="5">
         <f>IF(E15&lt;2,"积累中",IF(I15&gt;=0.01,"上涨",IF(I15&lt;=-0.01,"下降","平稳")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Kingfoodmart</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Vĩnh Tân</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>猪排</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>胡志明市/Kingfoodmart默认门店</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>197500</v>
+      </c>
+      <c r="G16" s="7" t="n">
+        <v>197500</v>
+      </c>
+      <c r="H16" s="7" t="n">
+        <v>197500</v>
+      </c>
+      <c r="I16" s="9">
+        <f>IF(E16&lt;2,"",G16/F16-1)</f>
+        <v/>
+      </c>
+      <c r="J16" s="5">
+        <f>IF(E16&lt;2,"积累中",IF(I16&gt;=0.01,"上涨",IF(I16&lt;=-0.01,"下降","平稳")))</f>
         <v/>
       </c>
     </row>
@@ -1982,7 +2091,7 @@
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="I5:I15">
+  <conditionalFormatting sqref="I5:I16">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="1">
       <formula>0.01</formula>
     </cfRule>
@@ -2181,7 +2290,7 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-11
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-11</t>
+          <t>越南猪肉零售价格日报｜2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 05:20。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 05:24。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>10条在售商品</t>
+          <t>8条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-11</t>
+          <t>越南猪肉零售明细｜2026-08-12</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Vĩnh Tân 400g</t>
+          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1112,13 +1112,13 @@
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>77000</v>
+        <v>38000</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>192500</v>
+        <v>190000</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-400g-1-khay-63124</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
@@ -1296,12 +1296,12 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>肩肉</t>
+          <t>小排</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI Thịt Nạc vai heo (S)</t>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1310,13 +1310,13 @@
         </is>
       </c>
       <c r="I12" s="7" t="n">
-        <v>440</v>
+        <v>431</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>74316</v>
+        <v>124085</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>168900</v>
+        <v>287900</v>
       </c>
       <c r="L12" s="7" t="n"/>
       <c r="M12" s="7">
@@ -1330,139 +1330,7 @@
       </c>
       <c r="O12" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>小排</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I13" s="7" t="n">
-        <v>431</v>
-      </c>
-      <c r="J13" s="7" t="n">
-        <v>124085</v>
-      </c>
-      <c r="K13" s="7" t="n">
-        <v>287900</v>
-      </c>
-      <c r="L13" s="7" t="n"/>
-      <c r="M13" s="7">
-        <f>IF(L13&lt;&gt;"",L13,K13)</f>
-        <v/>
-      </c>
-      <c r="N13" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O13" s="8" t="inlineStr">
-        <is>
           <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>五花肉</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I14" s="7" t="n">
-        <v>385</v>
-      </c>
-      <c r="J14" s="7" t="n">
-        <v>76962</v>
-      </c>
-      <c r="K14" s="7" t="n">
-        <v>199900</v>
-      </c>
-      <c r="L14" s="7" t="n"/>
-      <c r="M14" s="7">
-        <f>IF(L14&lt;&gt;"",L14,K14)</f>
-        <v/>
-      </c>
-      <c r="N14" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O14" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1339,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M14">
+  <conditionalFormatting sqref="M5:M12">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1488,8 +1356,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1604,7 +1470,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1688,7 +1554,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1856,7 +1722,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1898,7 +1764,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -1940,7 +1806,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -1949,7 +1815,7 @@
         <v>138889</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>127778</v>
+        <v>138889</v>
       </c>
       <c r="I13" s="9">
         <f>IF(E13&lt;2,"",G13/F13-1)</f>
@@ -1982,7 +1848,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>165000</v>
@@ -2024,13 +1890,13 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>192500</v>
+        <v>190000</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>190000</v>
@@ -2066,7 +1932,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>
@@ -2258,7 +2124,7 @@
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-400g-1-khay-63124</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
@@ -2290,7 +2156,7 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-12
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,7 +547,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-12</t>
+          <t>越南猪肉零售价格日报｜2026-08-13</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-12</t>
+          <t>越南猪肉零售明细｜2026-08-13</t>
         </is>
       </c>
     </row>
@@ -1470,7 +1470,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1554,7 +1554,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1722,7 +1722,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1764,7 +1764,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -1806,7 +1806,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -1848,7 +1848,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>165000</v>
@@ -1890,7 +1890,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
@@ -1932,7 +1932,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-13
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,7 +547,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-13</t>
+          <t>越南猪肉零售价格日报｜2026-08-14</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>8条在售商品</t>
+          <t>9条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O12"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-13</t>
+          <t>越南猪肉零售明细｜2026-08-14</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1000,7 @@
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/sap-mo-ban-cot-let-meatcool-tui-900g-ol341387</t>
+          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g-ol341387</t>
         </is>
       </c>
     </row>
@@ -1331,6 +1331,72 @@
       <c r="O12" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>全国渠道</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>WinMart默认门店（待固定城市）</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>WinMart</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Masan</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>MEATDeli</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>五花肉</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>冷鲜</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>385</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>76962</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>199900</v>
+      </c>
+      <c r="L13" s="7" t="n"/>
+      <c r="M13" s="7">
+        <f>IF(L13&lt;&gt;"",L13,K13)</f>
+        <v/>
+      </c>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>中：官方交易页，但尚未固定配送门店</t>
+        </is>
+      </c>
+      <c r="O13" s="8" t="inlineStr">
+        <is>
+          <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1405,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M12">
+  <conditionalFormatting sqref="M5:M13">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1356,6 +1422,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1470,7 +1537,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1512,7 +1579,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1554,7 +1621,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1722,7 +1789,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1764,7 +1831,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -1806,7 +1873,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -1848,7 +1915,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>165000</v>
@@ -1890,7 +1957,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
@@ -1932,7 +1999,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-14
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-14</t>
+          <t>越南猪肉零售价格日报｜2026-08-15</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 05:24。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 04:58。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>9条在售商品</t>
+          <t>6条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-14</t>
+          <t>越南猪肉零售明细｜2026-08-15</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1000,7 @@
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g-ol341387</t>
+          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -1022,22 +1022,22 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Thịt đùi Meatcool túi 900g</t>
+          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1046,13 +1046,13 @@
         </is>
       </c>
       <c r="I8" s="7" t="n">
-        <v>900</v>
+        <v>200</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>125000</v>
+        <v>38000</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>138889</v>
+        <v>190000</v>
       </c>
       <c r="L8" s="7" t="n"/>
       <c r="M8" s="7">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
@@ -1098,12 +1098,12 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
+          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1112,13 +1112,13 @@
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>38000</v>
+        <v>79000</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>190000</v>
+        <v>197500</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
@@ -1132,44 +1132,44 @@
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
         </is>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>小排</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -1178,13 +1178,13 @@
         </is>
       </c>
       <c r="I10" s="7" t="n">
-        <v>400</v>
+        <v>431</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>79000</v>
+        <v>124085</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>197500</v>
+        <v>287900</v>
       </c>
       <c r="L10" s="7" t="n"/>
       <c r="M10" s="7">
@@ -1193,210 +1193,12 @@
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O10" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>南部</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Kingfoodmart</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Vĩnh Tân</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>Vĩnh Tân</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>后腿肉</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I11" s="7" t="n">
-        <v>200</v>
-      </c>
-      <c r="J11" s="7" t="n">
-        <v>33000</v>
-      </c>
-      <c r="K11" s="7" t="n">
-        <v>165000</v>
-      </c>
-      <c r="L11" s="7" t="n"/>
-      <c r="M11" s="7">
-        <f>IF(L11&lt;&gt;"",L11,K11)</f>
-        <v/>
-      </c>
-      <c r="N11" s="5" t="inlineStr">
-        <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
-        </is>
-      </c>
-      <c r="O11" s="8" t="inlineStr">
-        <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>小排</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I12" s="7" t="n">
-        <v>431</v>
-      </c>
-      <c r="J12" s="7" t="n">
-        <v>124085</v>
-      </c>
-      <c r="K12" s="7" t="n">
-        <v>287900</v>
-      </c>
-      <c r="L12" s="7" t="n"/>
-      <c r="M12" s="7">
-        <f>IF(L12&lt;&gt;"",L12,K12)</f>
-        <v/>
-      </c>
-      <c r="N12" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O12" s="8" t="inlineStr">
-        <is>
           <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>五花肉</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I13" s="7" t="n">
-        <v>385</v>
-      </c>
-      <c r="J13" s="7" t="n">
-        <v>76962</v>
-      </c>
-      <c r="K13" s="7" t="n">
-        <v>199900</v>
-      </c>
-      <c r="L13" s="7" t="n"/>
-      <c r="M13" s="7">
-        <f>IF(L13&lt;&gt;"",L13,K13)</f>
-        <v/>
-      </c>
-      <c r="N13" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O13" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1207,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M13">
+  <conditionalFormatting sqref="M5:M10">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1420,9 +1222,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1537,7 +1336,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1621,7 +1420,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1831,7 +1630,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -1873,7 +1672,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -1957,7 +1756,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
@@ -1999,7 +1798,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-15
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-15</t>
+          <t>越南猪肉零售价格日报｜2026-08-16</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 04:58。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 04:56。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>6条在售商品</t>
+          <t>8条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -632,7 +632,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>10组</t>
+          <t>11组</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-15</t>
+          <t>越南猪肉零售明细｜2026-08-16</t>
         </is>
       </c>
     </row>
@@ -1022,22 +1022,22 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
+          <t>Thịt đùi Meatcool túi 900g</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1046,13 +1046,13 @@
         </is>
       </c>
       <c r="I8" s="7" t="n">
-        <v>200</v>
+        <v>900</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>38000</v>
+        <v>125000</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>190000</v>
+        <v>138889</v>
       </c>
       <c r="L8" s="7" t="n"/>
       <c r="M8" s="7">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
+          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -1098,12 +1098,12 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
+          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1112,13 +1112,13 @@
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>79000</v>
+        <v>38000</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>197500</v>
+        <v>190000</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
@@ -1132,44 +1132,44 @@
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>全国渠道</t>
+          <t>南部</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>WinMart默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>WinMart</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Masan</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>MEATDeli</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>小排</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
+          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -1178,13 +1178,13 @@
         </is>
       </c>
       <c r="I10" s="7" t="n">
-        <v>431</v>
+        <v>400</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>124085</v>
+        <v>79000</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>287900</v>
+        <v>197500</v>
       </c>
       <c r="L10" s="7" t="n"/>
       <c r="M10" s="7">
@@ -1193,10 +1193,142 @@
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+        </is>
+      </c>
+      <c r="O10" s="8" t="inlineStr">
+        <is>
+          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>全国渠道</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>WinMart默认门店（待固定城市）</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>WinMart</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Masan</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>MEATDeli</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>肩肉</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>MEATDELI Thịt Nạc vai heo (S)</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>冷鲜</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="n">
+        <v>440</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>74316</v>
+      </c>
+      <c r="K11" s="7" t="n">
+        <v>168900</v>
+      </c>
+      <c r="L11" s="7" t="n"/>
+      <c r="M11" s="7">
+        <f>IF(L11&lt;&gt;"",L11,K11)</f>
+        <v/>
+      </c>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
           <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
-      <c r="O10" s="8" t="inlineStr">
+      <c r="O11" s="8" t="inlineStr">
+        <is>
+          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>全国渠道</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>WinMart默认门店（待固定城市）</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>WinMart</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Masan</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>MEATDeli</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>小排</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>冷鲜</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="n">
+        <v>431</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>124085</v>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>287900</v>
+      </c>
+      <c r="L12" s="7" t="n"/>
+      <c r="M12" s="7">
+        <f>IF(L12&lt;&gt;"",L12,K12)</f>
+        <v/>
+      </c>
+      <c r="N12" s="5" t="inlineStr">
+        <is>
+          <t>中：官方交易页，但尚未固定配送门店</t>
+        </is>
+      </c>
+      <c r="O12" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
@@ -1207,7 +1339,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M10">
+  <conditionalFormatting sqref="M5:M12">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1222,6 +1354,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1336,7 +1470,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1420,7 +1554,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1504,7 +1638,7 @@
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>168900</v>
@@ -1588,7 +1722,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1630,7 +1764,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -1672,7 +1806,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -1756,7 +1890,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
@@ -1798,7 +1932,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>
@@ -2022,7 +2156,7 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-16
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,7 +547,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-16</t>
+          <t>越南猪肉零售价格日报｜2026-08-17</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-16</t>
+          <t>越南猪肉零售明细｜2026-08-17</t>
         </is>
       </c>
     </row>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g-ol341387</t>
         </is>
       </c>
     </row>
@@ -1205,37 +1205,37 @@
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>全国渠道</t>
+          <t>南部</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>WinMart默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>WinMart</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Masan</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>MEATDeli</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>肩肉</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI Thịt Nạc vai heo (S)</t>
+          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1244,13 +1244,13 @@
         </is>
       </c>
       <c r="I11" s="7" t="n">
-        <v>440</v>
+        <v>200</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>74316</v>
+        <v>33000</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>168900</v>
+        <v>165000</v>
       </c>
       <c r="L11" s="7" t="n"/>
       <c r="M11" s="7">
@@ -1259,12 +1259,12 @@
       </c>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
         </is>
       </c>
       <c r="O11" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
@@ -1470,7 +1470,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1554,7 +1554,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1722,7 +1722,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1764,7 +1764,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -1806,7 +1806,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -1848,7 +1848,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>165000</v>
@@ -1890,7 +1890,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
@@ -1932,7 +1932,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>
@@ -2156,7 +2156,7 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-17
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-17</t>
+          <t>越南猪肉零售价格日报｜2026-08-18</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 04:56。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 04:59。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>8条在售商品</t>
+          <t>9条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -632,7 +632,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>11组</t>
+          <t>12组</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O12"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-17</t>
+          <t>越南猪肉零售明细｜2026-08-18</t>
         </is>
       </c>
     </row>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g-ol341387</t>
+          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -1331,6 +1331,72 @@
       <c r="O12" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>全国渠道</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>WinMart默认门店（待固定城市）</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>WinMart</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Masan</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>MEATDeli</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>梅花肉</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>冷鲜</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>400</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>81960</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>204900</v>
+      </c>
+      <c r="L13" s="7" t="n"/>
+      <c r="M13" s="7">
+        <f>IF(L13&lt;&gt;"",L13,K13)</f>
+        <v/>
+      </c>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>中：官方交易页，但尚未固定配送门店</t>
+        </is>
+      </c>
+      <c r="O13" s="8" t="inlineStr">
+        <is>
+          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1405,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M12">
+  <conditionalFormatting sqref="M5:M13">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1356,6 +1422,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1470,7 +1537,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1554,7 +1621,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1596,7 +1663,7 @@
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>204900</v>
@@ -1722,7 +1789,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1764,7 +1831,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -1806,7 +1873,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -1848,7 +1915,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>165000</v>
@@ -1890,7 +1957,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
@@ -1932,7 +1999,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-18
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-18</t>
+          <t>越南猪肉零售价格日报｜2026-08-19</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 04:59。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 04:57。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-18</t>
+          <t>越南猪肉零售明细｜2026-08-19</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
+          <t>Nạc dăm heo Vĩnh Tân 400g</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1112,13 +1112,13 @@
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>38000</v>
+        <v>77000</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>190000</v>
+        <v>192500</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-400g-1-khay-63124</t>
         </is>
       </c>
     </row>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -1376,13 +1376,13 @@
         </is>
       </c>
       <c r="I13" s="7" t="n">
-        <v>400</v>
+        <v>385</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>81960</v>
+        <v>76962</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>204900</v>
+        <v>199900</v>
       </c>
       <c r="L13" s="7" t="n"/>
       <c r="M13" s="7">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="O13" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
+          <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
       </c>
     </row>
@@ -1537,7 +1537,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1579,7 +1579,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1621,7 +1621,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1789,7 +1789,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1831,7 +1831,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -1873,7 +1873,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -1915,7 +1915,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>165000</v>
@@ -1957,13 +1957,13 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>190000</v>
+        <v>192500</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>190000</v>
@@ -1999,7 +1999,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>
@@ -2191,7 +2191,7 @@
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-400g-1-khay-63124</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-19
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-19</t>
+          <t>越南猪肉零售价格日报｜2026-08-20</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 04:57。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 05:00。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-19</t>
+          <t>越南猪肉零售明细｜2026-08-20</t>
         </is>
       </c>
     </row>
@@ -1537,7 +1537,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1579,7 +1579,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1621,7 +1621,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1789,7 +1789,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1831,7 +1831,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -1873,7 +1873,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -1915,7 +1915,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>165000</v>
@@ -1957,7 +1957,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
@@ -1999,7 +1999,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-20
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-20</t>
+          <t>越南猪肉零售价格日报｜2026-08-21</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 05:00。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 05:01。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>9条在售商品</t>
+          <t>8条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-20</t>
+          <t>越南猪肉零售明细｜2026-08-21</t>
         </is>
       </c>
     </row>
@@ -956,22 +956,22 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
+          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -980,13 +980,13 @@
         </is>
       </c>
       <c r="I7" s="7" t="n">
-        <v>900</v>
+        <v>200</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>125000</v>
+        <v>38000</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>138889</v>
+        <v>190000</v>
       </c>
       <c r="L7" s="7" t="n"/>
       <c r="M7" s="7">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
@@ -1022,22 +1022,22 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Thịt đùi Meatcool túi 900g</t>
+          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1046,13 +1046,13 @@
         </is>
       </c>
       <c r="I8" s="7" t="n">
-        <v>900</v>
+        <v>400</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>125000</v>
+        <v>79000</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>138889</v>
+        <v>197500</v>
       </c>
       <c r="L8" s="7" t="n"/>
       <c r="M8" s="7">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
         </is>
       </c>
     </row>
@@ -1098,12 +1098,12 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Vĩnh Tân 400g</t>
+          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1112,13 +1112,13 @@
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>77000</v>
+        <v>33000</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>192500</v>
+        <v>165000</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
@@ -1132,44 +1132,44 @@
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-400g-1-khay-63124</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>小排</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -1178,13 +1178,13 @@
         </is>
       </c>
       <c r="I10" s="7" t="n">
-        <v>400</v>
+        <v>431</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>79000</v>
+        <v>124085</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>197500</v>
+        <v>287900</v>
       </c>
       <c r="L10" s="7" t="n"/>
       <c r="M10" s="7">
@@ -1193,49 +1193,49 @@
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O10" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
+          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1244,13 +1244,13 @@
         </is>
       </c>
       <c r="I11" s="7" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>33000</v>
+        <v>81960</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>165000</v>
+        <v>204900</v>
       </c>
       <c r="L11" s="7" t="n"/>
       <c r="M11" s="7">
@@ -1259,12 +1259,12 @@
       </c>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O11" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
+          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
         </is>
       </c>
     </row>
@@ -1296,12 +1296,12 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>小排</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1310,13 +1310,13 @@
         </is>
       </c>
       <c r="I12" s="7" t="n">
-        <v>431</v>
+        <v>385</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>124085</v>
+        <v>76962</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>287900</v>
+        <v>199900</v>
       </c>
       <c r="L12" s="7" t="n"/>
       <c r="M12" s="7">
@@ -1329,72 +1329,6 @@
         </is>
       </c>
       <c r="O12" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>五花肉</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I13" s="7" t="n">
-        <v>385</v>
-      </c>
-      <c r="J13" s="7" t="n">
-        <v>76962</v>
-      </c>
-      <c r="K13" s="7" t="n">
-        <v>199900</v>
-      </c>
-      <c r="L13" s="7" t="n"/>
-      <c r="M13" s="7">
-        <f>IF(L13&lt;&gt;"",L13,K13)</f>
-        <v/>
-      </c>
-      <c r="N13" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O13" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
@@ -1405,7 +1339,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M13">
+  <conditionalFormatting sqref="M5:M12">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1422,7 +1356,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1537,7 +1470,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1579,7 +1512,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1621,7 +1554,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1663,7 +1596,7 @@
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>204900</v>
@@ -1831,7 +1764,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -1915,7 +1848,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>165000</v>
@@ -1957,13 +1890,13 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>192500</v>
+        <v>190000</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>190000</v>
@@ -1999,7 +1932,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>
@@ -2191,7 +2124,7 @@
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-400g-1-khay-63124</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-21
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-21</t>
+          <t>越南猪肉零售价格日报｜2026-08-22</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 05:01。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 04:59。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>8条在售商品</t>
+          <t>6条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -610,12 +610,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>4个</t>
+          <t>3个</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>BAF、MEATDeli、Meatcool、Vĩnh Tân</t>
+          <t>MEATDeli、Meatcool、Vĩnh Tân</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O12"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-21</t>
+          <t>越南猪肉零售明细｜2026-08-22</t>
         </is>
       </c>
     </row>
@@ -890,22 +890,22 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>BAF</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>BAF</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo BAF khay 300g</t>
+          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -914,13 +914,13 @@
         </is>
       </c>
       <c r="I6" s="7" t="n">
-        <v>300</v>
+        <v>900</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>74000</v>
+        <v>125000</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>246667</v>
+        <v>138889</v>
       </c>
       <c r="L6" s="7" t="n"/>
       <c r="M6" s="7">
@@ -934,7 +934,7 @@
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -956,22 +956,22 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
+          <t>Thịt đùi Meatcool túi 900g</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -980,13 +980,13 @@
         </is>
       </c>
       <c r="I7" s="7" t="n">
-        <v>200</v>
+        <v>900</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>38000</v>
+        <v>125000</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>190000</v>
+        <v>138889</v>
       </c>
       <c r="L7" s="7" t="n"/>
       <c r="M7" s="7">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
+          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -1032,12 +1032,12 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
+          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1046,13 +1046,13 @@
         </is>
       </c>
       <c r="I8" s="7" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>79000</v>
+        <v>38000</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>197500</v>
+        <v>190000</v>
       </c>
       <c r="L8" s="7" t="n"/>
       <c r="M8" s="7">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
@@ -1098,12 +1098,12 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
+          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1112,13 +1112,13 @@
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>33000</v>
+        <v>79000</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>165000</v>
+        <v>197500</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
         </is>
       </c>
     </row>
@@ -1199,138 +1199,6 @@
       <c r="O10" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>梅花肉</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I11" s="7" t="n">
-        <v>400</v>
-      </c>
-      <c r="J11" s="7" t="n">
-        <v>81960</v>
-      </c>
-      <c r="K11" s="7" t="n">
-        <v>204900</v>
-      </c>
-      <c r="L11" s="7" t="n"/>
-      <c r="M11" s="7">
-        <f>IF(L11&lt;&gt;"",L11,K11)</f>
-        <v/>
-      </c>
-      <c r="N11" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O11" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>五花肉</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I12" s="7" t="n">
-        <v>385</v>
-      </c>
-      <c r="J12" s="7" t="n">
-        <v>76962</v>
-      </c>
-      <c r="K12" s="7" t="n">
-        <v>199900</v>
-      </c>
-      <c r="L12" s="7" t="n"/>
-      <c r="M12" s="7">
-        <f>IF(L12&lt;&gt;"",L12,K12)</f>
-        <v/>
-      </c>
-      <c r="N12" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O12" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1207,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M12">
+  <conditionalFormatting sqref="M5:M10">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1354,8 +1222,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1554,7 +1420,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1722,7 +1588,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1764,7 +1630,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -1806,7 +1672,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -1890,7 +1756,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
@@ -1932,7 +1798,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>
@@ -1975,7 +1841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2072,7 +1938,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>BAF / BAF</t>
+          <t>Vĩnh Tân / Vĩnh Tân</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -2092,24 +1958,24 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
     <row r="7" ht="58" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân / Vĩnh Tân</t>
+          <t>Masan / MEATDeli</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>A-零售交易页</t>
+          <t>A-官方交易页</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -2119,42 +1985,10 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="58" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Masan / MEATDeli</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>A-官方交易页</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>实际价/kg = 促销价/kg（如有），否则常规价/kg；包装价÷重量(kg)用于交叉核验。</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
@@ -2169,7 +2003,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-22
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-22</t>
+          <t>越南猪肉零售价格日报｜2026-08-23</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 04:59。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 04:57。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>6条在售商品</t>
+          <t>9条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -610,12 +610,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>3个</t>
+          <t>4个</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>MEATDeli、Meatcool、Vĩnh Tân</t>
+          <t>BAF、MEATDeli、Meatcool、Vĩnh Tân</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-22</t>
+          <t>越南猪肉零售明细｜2026-08-23</t>
         </is>
       </c>
     </row>
@@ -890,22 +890,22 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>BAF</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>BAF</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
+          <t>Nạc dăm heo BAF khay 300g</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -914,13 +914,13 @@
         </is>
       </c>
       <c r="I6" s="7" t="n">
-        <v>900</v>
+        <v>300</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>125000</v>
+        <v>74000</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>138889</v>
+        <v>246667</v>
       </c>
       <c r="L6" s="7" t="n"/>
       <c r="M6" s="7">
@@ -934,7 +934,7 @@
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
         </is>
       </c>
     </row>
@@ -966,12 +966,12 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Thịt đùi Meatcool túi 900g</t>
+          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -1022,22 +1022,22 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
+          <t>Thịt đùi Meatcool túi 900g</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1046,13 +1046,13 @@
         </is>
       </c>
       <c r="I8" s="7" t="n">
-        <v>200</v>
+        <v>900</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>38000</v>
+        <v>125000</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>190000</v>
+        <v>138889</v>
       </c>
       <c r="L8" s="7" t="n"/>
       <c r="M8" s="7">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
+          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -1098,12 +1098,12 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
+          <t>Nạc dăm heo Vĩnh Tân 400g</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1115,10 +1115,10 @@
         <v>400</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>79000</v>
+        <v>77000</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>197500</v>
+        <v>192500</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
@@ -1132,44 +1132,44 @@
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-400g-1-khay-63124</t>
         </is>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>全国渠道</t>
+          <t>南部</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>WinMart默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>WinMart</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Masan</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>MEATDeli</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>小排</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
+          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -1178,13 +1178,13 @@
         </is>
       </c>
       <c r="I10" s="7" t="n">
-        <v>431</v>
+        <v>400</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>124085</v>
+        <v>79000</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>287900</v>
+        <v>197500</v>
       </c>
       <c r="L10" s="7" t="n"/>
       <c r="M10" s="7">
@@ -1193,12 +1193,210 @@
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+        </is>
+      </c>
+      <c r="O10" s="8" t="inlineStr">
+        <is>
+          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>南部</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>胡志明市/Kingfoodmart默认门店</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Kingfoodmart</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Vĩnh Tân</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Vĩnh Tân</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>后腿肉</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>冷鲜</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>33000</v>
+      </c>
+      <c r="K11" s="7" t="n">
+        <v>165000</v>
+      </c>
+      <c r="L11" s="7" t="n"/>
+      <c r="M11" s="7">
+        <f>IF(L11&lt;&gt;"",L11,K11)</f>
+        <v/>
+      </c>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+        </is>
+      </c>
+      <c r="O11" s="8" t="inlineStr">
+        <is>
+          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>全国渠道</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>WinMart默认门店（待固定城市）</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>WinMart</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Masan</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>MEATDeli</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>小排</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>冷鲜</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="n">
+        <v>431</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>124085</v>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>287900</v>
+      </c>
+      <c r="L12" s="7" t="n"/>
+      <c r="M12" s="7">
+        <f>IF(L12&lt;&gt;"",L12,K12)</f>
+        <v/>
+      </c>
+      <c r="N12" s="5" t="inlineStr">
+        <is>
           <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
-      <c r="O10" s="8" t="inlineStr">
+      <c r="O12" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>全国渠道</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>WinMart默认门店（待固定城市）</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>WinMart</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Masan</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>MEATDeli</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>梅花肉</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>冷鲜</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>400</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>81960</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>204900</v>
+      </c>
+      <c r="L13" s="7" t="n"/>
+      <c r="M13" s="7">
+        <f>IF(L13&lt;&gt;"",L13,K13)</f>
+        <v/>
+      </c>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>中：官方交易页，但尚未固定配送门店</t>
+        </is>
+      </c>
+      <c r="O13" s="8" t="inlineStr">
+        <is>
+          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
         </is>
       </c>
     </row>
@@ -1207,7 +1405,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M10">
+  <conditionalFormatting sqref="M5:M13">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1222,6 +1420,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1336,7 +1537,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1420,7 +1621,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1462,7 +1663,7 @@
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>204900</v>
@@ -1588,7 +1789,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1630,7 +1831,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -1672,7 +1873,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -1714,7 +1915,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>165000</v>
@@ -1756,13 +1957,13 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>190000</v>
+        <v>192500</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>190000</v>
@@ -1798,7 +1999,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>
@@ -1841,7 +2042,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1938,7 +2139,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân / Vĩnh Tân</t>
+          <t>BAF / BAF</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -1958,37 +2159,69 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
         </is>
       </c>
     </row>
     <row r="7" ht="58" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
+          <t>Kingfoodmart</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Vĩnh Tân / Vĩnh Tân</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>A-零售交易页</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>实际价/kg = 促销价/kg（如有），否则常规价/kg；包装价÷重量(kg)用于交叉核验。</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-400g-1-khay-63124</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="58" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
           <t>WinMart</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Masan / MEATDeli</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>A-官方交易页</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>实际价/kg = 促销价/kg（如有），否则常规价/kg；包装价÷重量(kg)用于交叉核验。</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
@@ -2003,6 +2236,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-23
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,7 +547,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-23</t>
+          <t>越南猪肉零售价格日报｜2026-08-24</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>9条在售商品</t>
+          <t>8条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-23</t>
+          <t>越南猪肉零售明细｜2026-08-24</t>
         </is>
       </c>
     </row>
@@ -1331,72 +1331,6 @@
       <c r="O12" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>梅花肉</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I13" s="7" t="n">
-        <v>400</v>
-      </c>
-      <c r="J13" s="7" t="n">
-        <v>81960</v>
-      </c>
-      <c r="K13" s="7" t="n">
-        <v>204900</v>
-      </c>
-      <c r="L13" s="7" t="n"/>
-      <c r="M13" s="7">
-        <f>IF(L13&lt;&gt;"",L13,K13)</f>
-        <v/>
-      </c>
-      <c r="N13" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O13" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1339,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M13">
+  <conditionalFormatting sqref="M5:M12">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1422,7 +1356,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1537,7 +1470,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1621,7 +1554,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1789,7 +1722,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1831,7 +1764,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -1873,7 +1806,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -1915,7 +1848,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>165000</v>
@@ -1957,7 +1890,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
@@ -1999,7 +1932,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-24
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-24</t>
+          <t>越南猪肉零售价格日报｜2026-08-25</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 04:57。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 05:01。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-24</t>
+          <t>越南猪肉零售明细｜2026-08-25</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Vĩnh Tân 400g</t>
+          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1112,13 +1112,13 @@
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>77000</v>
+        <v>38000</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>192500</v>
+        <v>190000</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-400g-1-khay-63124</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
@@ -1470,7 +1470,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1554,7 +1554,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1722,7 +1722,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1764,7 +1764,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -1806,7 +1806,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -1848,7 +1848,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>165000</v>
@@ -1890,13 +1890,13 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>192500</v>
+        <v>190000</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>190000</v>
@@ -1932,7 +1932,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>
@@ -2124,7 +2124,7 @@
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-400g-1-khay-63124</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-25
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-25</t>
+          <t>越南猪肉零售价格日报｜2026-08-26</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 05:01。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 05:00。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>8条在售商品</t>
+          <t>10条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O12"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-25</t>
+          <t>越南猪肉零售明细｜2026-08-26</t>
         </is>
       </c>
     </row>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g-ol341387</t>
         </is>
       </c>
     </row>
@@ -1296,12 +1296,12 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>小排</t>
+          <t>肩肉</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
+          <t>MEATDELI Thịt Nạc vai heo (S)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1310,13 +1310,13 @@
         </is>
       </c>
       <c r="I12" s="7" t="n">
-        <v>431</v>
+        <v>440</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>124085</v>
+        <v>74316</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>287900</v>
+        <v>168900</v>
       </c>
       <c r="L12" s="7" t="n"/>
       <c r="M12" s="7">
@@ -1330,7 +1330,139 @@
       </c>
       <c r="O12" s="8" t="inlineStr">
         <is>
+          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>全国渠道</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>WinMart默认门店（待固定城市）</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>WinMart</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Masan</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>MEATDeli</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>小排</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>冷鲜</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>431</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>124085</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>287900</v>
+      </c>
+      <c r="L13" s="7" t="n"/>
+      <c r="M13" s="7">
+        <f>IF(L13&lt;&gt;"",L13,K13)</f>
+        <v/>
+      </c>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>中：官方交易页，但尚未固定配送门店</t>
+        </is>
+      </c>
+      <c r="O13" s="8" t="inlineStr">
+        <is>
           <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>全国渠道</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>WinMart默认门店（待固定城市）</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>WinMart</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Masan</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>MEATDeli</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>五花肉</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>冷鲜</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>385</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>76962</v>
+      </c>
+      <c r="K14" s="7" t="n">
+        <v>199900</v>
+      </c>
+      <c r="L14" s="7" t="n"/>
+      <c r="M14" s="7">
+        <f>IF(L14&lt;&gt;"",L14,K14)</f>
+        <v/>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>中：官方交易页，但尚未固定配送门店</t>
+        </is>
+      </c>
+      <c r="O14" s="8" t="inlineStr">
+        <is>
+          <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1471,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M12">
+  <conditionalFormatting sqref="M5:M14">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1356,6 +1488,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1470,7 +1604,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1512,7 +1646,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1554,7 +1688,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1638,7 +1772,7 @@
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>168900</v>
@@ -1722,7 +1856,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1764,7 +1898,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -1806,7 +1940,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -1848,7 +1982,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>165000</v>
@@ -1890,7 +2024,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
@@ -1932,7 +2066,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>
@@ -2156,7 +2290,7 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-27
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-26</t>
+          <t>越南猪肉零售价格日报｜2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 05:00。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 08:05。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>10条在售商品</t>
+          <t>9条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-26</t>
+          <t>越南猪肉零售明细｜2026-08-27</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1000,7 @@
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g-ol341387</t>
         </is>
       </c>
     </row>
@@ -1296,12 +1296,12 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>肩肉</t>
+          <t>小排</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI Thịt Nạc vai heo (S)</t>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1310,13 +1310,13 @@
         </is>
       </c>
       <c r="I12" s="7" t="n">
-        <v>440</v>
+        <v>431</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>74316</v>
+        <v>124085</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>168900</v>
+        <v>287900</v>
       </c>
       <c r="L12" s="7" t="n"/>
       <c r="M12" s="7">
@@ -1330,7 +1330,7 @@
       </c>
       <c r="O12" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>
@@ -1362,12 +1362,12 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>小排</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -1376,13 +1376,13 @@
         </is>
       </c>
       <c r="I13" s="7" t="n">
-        <v>431</v>
+        <v>385</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>124085</v>
+        <v>76962</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>287900</v>
+        <v>199900</v>
       </c>
       <c r="L13" s="7" t="n"/>
       <c r="M13" s="7">
@@ -1395,72 +1395,6 @@
         </is>
       </c>
       <c r="O13" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>五花肉</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I14" s="7" t="n">
-        <v>385</v>
-      </c>
-      <c r="J14" s="7" t="n">
-        <v>76962</v>
-      </c>
-      <c r="K14" s="7" t="n">
-        <v>199900</v>
-      </c>
-      <c r="L14" s="7" t="n"/>
-      <c r="M14" s="7">
-        <f>IF(L14&lt;&gt;"",L14,K14)</f>
-        <v/>
-      </c>
-      <c r="N14" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O14" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
@@ -1471,7 +1405,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M14">
+  <conditionalFormatting sqref="M5:M13">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1489,7 +1423,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1604,7 +1537,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1646,7 +1579,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1688,7 +1621,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1856,7 +1789,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1898,7 +1831,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -1940,7 +1873,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -1982,7 +1915,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>165000</v>
@@ -2024,7 +1957,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
@@ -2066,7 +1999,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>
@@ -2290,7 +2223,7 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-28
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-27</t>
+          <t>越南猪肉零售价格日报｜2026-08-28</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 08:05。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 12:49。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>9条在售商品</t>
+          <t>8条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -610,12 +610,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>4个</t>
+          <t>3个</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>BAF、MEATDeli、Meatcool、Vĩnh Tân</t>
+          <t>MEATDeli、Meatcool、Vĩnh Tân</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-27</t>
+          <t>越南猪肉零售明细｜2026-08-28</t>
         </is>
       </c>
     </row>
@@ -832,12 +832,12 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Meatcool 360-440g</t>
+          <t>Ba rọi heo Meatcool 360-440g</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -849,13 +849,13 @@
         <v>400</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>90400</v>
+        <v>99600</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>226000</v>
+        <v>249000</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>192100</v>
+        <v>197500</v>
       </c>
       <c r="M5" s="7">
         <f>IF(L5&lt;&gt;"",L5,K5)</f>
@@ -868,7 +868,7 @@
       </c>
       <c r="O5" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-meatcool-400g</t>
+          <t>https://kingfoodmart.com/thit-heo/ba-roi-heo-meatcool-400g</t>
         </is>
       </c>
     </row>
@@ -890,22 +890,22 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>BAF</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>BAF</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo BAF khay 300g</t>
+          <t>Thịt đùi Meatcool túi 900g</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -914,13 +914,13 @@
         </is>
       </c>
       <c r="I6" s="7" t="n">
-        <v>300</v>
+        <v>900</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>74000</v>
+        <v>125000</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>246667</v>
+        <v>138889</v>
       </c>
       <c r="L6" s="7" t="n"/>
       <c r="M6" s="7">
@@ -934,7 +934,7 @@
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g-ol341387</t>
         </is>
       </c>
     </row>
@@ -971,7 +971,7 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
+          <t>Cốt lết heo Meatcool khay 300g</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -980,13 +980,13 @@
         </is>
       </c>
       <c r="I7" s="7" t="n">
-        <v>900</v>
+        <v>300</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>125000</v>
+        <v>35000</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>138889</v>
+        <v>116667</v>
       </c>
       <c r="L7" s="7" t="n"/>
       <c r="M7" s="7">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g-ol341387</t>
+          <t>https://kingfoodmart.com/thit-heo/cot-let-heo-meatcool-khay-300g</t>
         </is>
       </c>
     </row>
@@ -1022,22 +1022,22 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Thịt đùi Meatcool túi 900g</t>
+          <t>Ba rọi heo đặc biệt Vĩnh Tân 400g</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1046,13 +1046,13 @@
         </is>
       </c>
       <c r="I8" s="7" t="n">
-        <v>900</v>
+        <v>400</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>125000</v>
+        <v>89000</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>138889</v>
+        <v>222500</v>
       </c>
       <c r="L8" s="7" t="n"/>
       <c r="M8" s="7">
@@ -1066,44 +1066,44 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g-ol341387</t>
+          <t>https://kingfoodmart.com/thit-heo/ba-roi-heo-dac-biet-vinh-tan-400g-1-khay-63106</t>
         </is>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>肩肉</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
+          <t>MEATDELI Thịt Nạc vai heo (S)</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1112,13 +1112,13 @@
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>200</v>
+        <v>440</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>38000</v>
+        <v>74316</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>190000</v>
+        <v>168900</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
@@ -1127,49 +1127,49 @@
       </c>
       <c r="N9" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
+          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
         </is>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>小排</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -1178,13 +1178,13 @@
         </is>
       </c>
       <c r="I10" s="7" t="n">
-        <v>400</v>
+        <v>431</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>79000</v>
+        <v>124085</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>197500</v>
+        <v>287900</v>
       </c>
       <c r="L10" s="7" t="n"/>
       <c r="M10" s="7">
@@ -1193,49 +1193,49 @@
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O10" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
+          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1244,13 +1244,13 @@
         </is>
       </c>
       <c r="I11" s="7" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>33000</v>
+        <v>81960</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>165000</v>
+        <v>204900</v>
       </c>
       <c r="L11" s="7" t="n"/>
       <c r="M11" s="7">
@@ -1259,12 +1259,12 @@
       </c>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O11" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
+          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
         </is>
       </c>
     </row>
@@ -1296,12 +1296,12 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>小排</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1310,13 +1310,13 @@
         </is>
       </c>
       <c r="I12" s="7" t="n">
-        <v>431</v>
+        <v>385</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>124085</v>
+        <v>76962</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>287900</v>
+        <v>199900</v>
       </c>
       <c r="L12" s="7" t="n"/>
       <c r="M12" s="7">
@@ -1329,72 +1329,6 @@
         </is>
       </c>
       <c r="O12" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>五花肉</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I13" s="7" t="n">
-        <v>385</v>
-      </c>
-      <c r="J13" s="7" t="n">
-        <v>76962</v>
-      </c>
-      <c r="K13" s="7" t="n">
-        <v>199900</v>
-      </c>
-      <c r="L13" s="7" t="n"/>
-      <c r="M13" s="7">
-        <f>IF(L13&lt;&gt;"",L13,K13)</f>
-        <v/>
-      </c>
-      <c r="N13" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O13" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
@@ -1405,7 +1339,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M13">
+  <conditionalFormatting sqref="M5:M12">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1422,7 +1356,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1434,7 +1367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1579,7 +1512,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1621,7 +1554,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1663,7 +1596,7 @@
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>204900</v>
@@ -1705,7 +1638,7 @@
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>168900</v>
@@ -1747,13 +1680,13 @@
         </is>
       </c>
       <c r="E10" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F10" s="7" t="n">
         <v>195000</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>195000</v>
+        <v>197500</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>195000</v>
@@ -1789,7 +1722,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1873,13 +1806,13 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>138889</v>
+        <v>116667</v>
       </c>
       <c r="H13" s="7" t="n">
         <v>138889</v>
@@ -1906,7 +1839,7 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -1915,16 +1848,16 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>165000</v>
+        <v>222500</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>165000</v>
+        <v>222500</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>165000</v>
+        <v>222500</v>
       </c>
       <c r="I14" s="9">
         <f>IF(E14&lt;2,"",G14/F14-1)</f>
@@ -1948,7 +1881,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -1957,16 +1890,16 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>190000</v>
+        <v>165000</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>190000</v>
+        <v>165000</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>190000</v>
+        <v>165000</v>
       </c>
       <c r="I15" s="9">
         <f>IF(E15&lt;2,"",G15/F15-1)</f>
@@ -1990,7 +1923,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -2002,13 +1935,13 @@
         <v>27</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>197500</v>
+        <v>190000</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>197500</v>
+        <v>190000</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>197500</v>
+        <v>190000</v>
       </c>
       <c r="I16" s="9">
         <f>IF(E16&lt;2,"",G16/F16-1)</f>
@@ -2016,6 +1949,48 @@
       </c>
       <c r="J16" s="5">
         <f>IF(E16&lt;2,"积累中",IF(I16&gt;=0.01,"上涨",IF(I16&lt;=-0.01,"下降","平稳")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Kingfoodmart</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Vĩnh Tân</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>猪排</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>胡志明市/Kingfoodmart默认门店</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>27</v>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>197500</v>
+      </c>
+      <c r="G17" s="7" t="n">
+        <v>197500</v>
+      </c>
+      <c r="H17" s="7" t="n">
+        <v>197500</v>
+      </c>
+      <c r="I17" s="9">
+        <f>IF(E17&lt;2,"",G17/F17-1)</f>
+        <v/>
+      </c>
+      <c r="J17" s="5">
+        <f>IF(E17&lt;2,"积累中",IF(I17&gt;=0.01,"上涨",IF(I17&lt;=-0.01,"下降","平稳")))</f>
         <v/>
       </c>
     </row>
@@ -2024,7 +1999,7 @@
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="I5:I16">
+  <conditionalFormatting sqref="I5:I17">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="1">
       <formula>0.01</formula>
     </cfRule>
@@ -2042,7 +2017,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2127,7 +2102,7 @@
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-meatcool-400g</t>
+          <t>https://kingfoodmart.com/thit-heo/ba-roi-heo-meatcool-400g</t>
         </is>
       </c>
     </row>
@@ -2139,7 +2114,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>BAF / BAF</t>
+          <t>Vĩnh Tân / Vĩnh Tân</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -2159,24 +2134,24 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/ba-roi-heo-dac-biet-vinh-tan-400g-1-khay-63106</t>
         </is>
       </c>
     </row>
     <row r="7" ht="58" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân / Vĩnh Tân</t>
+          <t>Masan / MEATDeli</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>A-零售交易页</t>
+          <t>A-官方交易页</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -2186,44 +2161,12 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="58" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Masan / MEATDeli</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>A-官方交易页</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>实际价/kg = 促销价/kg（如有），否则常规价/kg；包装价÷重量(kg)用于交叉核验。</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
         </is>
       </c>
     </row>
@@ -2236,7 +2179,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-29
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-28</t>
+          <t>越南猪肉零售价格日报｜2026-08-29</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 12:49。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 10:23。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>8条在售商品</t>
+          <t>9条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>MEATDeli、Meatcool、Vĩnh Tân</t>
+          <t>BAF、MEATDeli、Meatcool</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O12"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-28</t>
+          <t>越南猪肉零售明细｜2026-08-29</t>
         </is>
       </c>
     </row>
@@ -890,22 +890,22 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>BAF</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>BAF</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Thịt đùi Meatcool túi 900g</t>
+          <t>Ba rọi heo BAF khay 300g</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -914,13 +914,13 @@
         </is>
       </c>
       <c r="I6" s="7" t="n">
-        <v>900</v>
+        <v>300</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>125000</v>
+        <v>79000</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>138889</v>
+        <v>263333</v>
       </c>
       <c r="L6" s="7" t="n"/>
       <c r="M6" s="7">
@@ -934,7 +934,7 @@
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g-ol341387</t>
+          <t>https://kingfoodmart.com/thit-heo/ba-roi-heo-baf-khay-300g-1-khay</t>
         </is>
       </c>
     </row>
@@ -956,22 +956,22 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>BAF</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>BAF</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Cốt lết heo Meatcool khay 300g</t>
+          <t>Nạc dăm heo BAF khay 300g</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -983,10 +983,10 @@
         <v>300</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>35000</v>
+        <v>74000</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>116667</v>
+        <v>246667</v>
       </c>
       <c r="L7" s="7" t="n"/>
       <c r="M7" s="7">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/cot-let-heo-meatcool-khay-300g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
         </is>
       </c>
     </row>
@@ -1022,22 +1022,22 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>五花肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Ba rọi heo đặc biệt Vĩnh Tân 400g</t>
+          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1046,13 +1046,13 @@
         </is>
       </c>
       <c r="I8" s="7" t="n">
-        <v>400</v>
+        <v>900</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>89000</v>
+        <v>125000</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>222500</v>
+        <v>138889</v>
       </c>
       <c r="L8" s="7" t="n"/>
       <c r="M8" s="7">
@@ -1066,44 +1066,44 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/ba-roi-heo-dac-biet-vinh-tan-400g-1-khay-63106</t>
+          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>全国渠道</t>
+          <t>南部</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>WinMart默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>WinMart</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Masan</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>MEATDeli</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>肩肉</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI Thịt Nạc vai heo (S)</t>
+          <t>Thịt đùi Meatcool túi 900g</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1112,13 +1112,13 @@
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>440</v>
+        <v>900</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>74316</v>
+        <v>125000</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>168900</v>
+        <v>138889</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
@@ -1127,12 +1127,12 @@
       </c>
       <c r="N9" s="5" t="inlineStr">
         <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
         </is>
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
+          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -1164,12 +1164,12 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>小排</t>
+          <t>肩肉</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
+          <t>MEATDELI Thịt Nạc vai heo (S)</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -1178,13 +1178,13 @@
         </is>
       </c>
       <c r="I10" s="7" t="n">
-        <v>431</v>
+        <v>440</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>124085</v>
+        <v>74316</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>287900</v>
+        <v>168900</v>
       </c>
       <c r="L10" s="7" t="n"/>
       <c r="M10" s="7">
@@ -1198,7 +1198,7 @@
       </c>
       <c r="O10" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
         </is>
       </c>
     </row>
@@ -1230,12 +1230,12 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>小排</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1244,13 +1244,13 @@
         </is>
       </c>
       <c r="I11" s="7" t="n">
-        <v>400</v>
+        <v>431</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>81960</v>
+        <v>124085</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>204900</v>
+        <v>287900</v>
       </c>
       <c r="L11" s="7" t="n"/>
       <c r="M11" s="7">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="O11" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>
@@ -1296,12 +1296,12 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>五花肉</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
+          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1310,13 +1310,13 @@
         </is>
       </c>
       <c r="I12" s="7" t="n">
-        <v>385</v>
+        <v>400</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>76962</v>
+        <v>81960</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>199900</v>
+        <v>204900</v>
       </c>
       <c r="L12" s="7" t="n"/>
       <c r="M12" s="7">
@@ -1329,6 +1329,72 @@
         </is>
       </c>
       <c r="O12" s="8" t="inlineStr">
+        <is>
+          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>全国渠道</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>WinMart默认门店（待固定城市）</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>WinMart</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Masan</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>MEATDeli</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>五花肉</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>冷鲜</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>385</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>76962</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>199900</v>
+      </c>
+      <c r="L13" s="7" t="n"/>
+      <c r="M13" s="7">
+        <f>IF(L13&lt;&gt;"",L13,K13)</f>
+        <v/>
+      </c>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>中：官方交易页，但尚未固定配送门店</t>
+        </is>
+      </c>
+      <c r="O13" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
@@ -1339,7 +1405,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M12">
+  <conditionalFormatting sqref="M5:M13">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1356,6 +1422,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1367,7 +1434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1461,7 +1528,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -1470,16 +1537,16 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>246667</v>
+        <v>263333</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>246667</v>
+        <v>263333</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>246667</v>
+        <v>263333</v>
       </c>
       <c r="I5" s="9">
         <f>IF(E5&lt;2,"",G5/F5-1)</f>
@@ -1493,35 +1560,35 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>WinMart</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>MEATDeli</t>
+          <t>BAF</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>五花肉</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>WinMart默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>199900</v>
+        <v>246667</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>199900</v>
+        <v>246667</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>199900</v>
+        <v>246667</v>
       </c>
       <c r="I6" s="9">
         <f>IF(E6&lt;2,"",G6/F6-1)</f>
@@ -1545,7 +1612,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>小排</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -1554,16 +1621,16 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>287900</v>
+        <v>199900</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>287900</v>
+        <v>199900</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>287900</v>
+        <v>199900</v>
       </c>
       <c r="I7" s="9">
         <f>IF(E7&lt;2,"",G7/F7-1)</f>
@@ -1587,7 +1654,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>小排</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -1596,16 +1663,16 @@
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>5</v>
+        <v>28</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>204900</v>
+        <v>287900</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>204900</v>
+        <v>287900</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>204900</v>
+        <v>287900</v>
       </c>
       <c r="I8" s="9">
         <f>IF(E8&lt;2,"",G8/F8-1)</f>
@@ -1629,7 +1696,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>肩肉</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -1638,16 +1705,16 @@
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>168900</v>
+        <v>204900</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>168900</v>
+        <v>204900</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>168900</v>
+        <v>204900</v>
       </c>
       <c r="I9" s="9">
         <f>IF(E9&lt;2,"",G9/F9-1)</f>
@@ -1661,35 +1728,35 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>五花肉</t>
+          <t>肩肉</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="E10" s="7" t="n">
         <v>5</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>195000</v>
+        <v>168900</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>197500</v>
+        <v>168900</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>195000</v>
+        <v>168900</v>
       </c>
       <c r="I10" s="9">
         <f>IF(E10&lt;2,"",G10/F10-1)</f>
@@ -1713,7 +1780,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -1722,16 +1789,16 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>138889</v>
+        <v>195000</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>138889</v>
+        <v>197500</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>138889</v>
+        <v>195000</v>
       </c>
       <c r="I11" s="9">
         <f>IF(E11&lt;2,"",G11/F11-1)</f>
@@ -1755,7 +1822,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -1764,16 +1831,16 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>192100</v>
+        <v>138889</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>192100</v>
+        <v>138889</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>192100</v>
+        <v>138889</v>
       </c>
       <c r="I12" s="9">
         <f>IF(E12&lt;2,"",G12/F12-1)</f>
@@ -1797,7 +1864,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -1806,16 +1873,16 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>138889</v>
+        <v>192100</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>116667</v>
+        <v>192100</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>138889</v>
+        <v>192100</v>
       </c>
       <c r="I13" s="9">
         <f>IF(E13&lt;2,"",G13/F13-1)</f>
@@ -1834,12 +1901,12 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>五花肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -1848,16 +1915,16 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>222500</v>
+        <v>138889</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>222500</v>
+        <v>138889</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>222500</v>
+        <v>138889</v>
       </c>
       <c r="I14" s="9">
         <f>IF(E14&lt;2,"",G14/F14-1)</f>
@@ -1881,7 +1948,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -1890,16 +1957,16 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>165000</v>
+        <v>222500</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>165000</v>
+        <v>222500</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>165000</v>
+        <v>222500</v>
       </c>
       <c r="I15" s="9">
         <f>IF(E15&lt;2,"",G15/F15-1)</f>
@@ -1923,7 +1990,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -1932,16 +1999,16 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>190000</v>
+        <v>165000</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>190000</v>
+        <v>165000</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>190000</v>
+        <v>165000</v>
       </c>
       <c r="I16" s="9">
         <f>IF(E16&lt;2,"",G16/F16-1)</f>
@@ -1965,7 +2032,7 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
@@ -1977,13 +2044,13 @@
         <v>27</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>197500</v>
+        <v>190000</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>197500</v>
+        <v>190000</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>197500</v>
+        <v>190000</v>
       </c>
       <c r="I17" s="9">
         <f>IF(E17&lt;2,"",G17/F17-1)</f>
@@ -1991,6 +2058,48 @@
       </c>
       <c r="J17" s="5">
         <f>IF(E17&lt;2,"积累中",IF(I17&gt;=0.01,"上涨",IF(I17&lt;=-0.01,"下降","平稳")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Kingfoodmart</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Vĩnh Tân</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>猪排</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>胡志明市/Kingfoodmart默认门店</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>27</v>
+      </c>
+      <c r="F18" s="7" t="n">
+        <v>197500</v>
+      </c>
+      <c r="G18" s="7" t="n">
+        <v>197500</v>
+      </c>
+      <c r="H18" s="7" t="n">
+        <v>197500</v>
+      </c>
+      <c r="I18" s="9">
+        <f>IF(E18&lt;2,"",G18/F18-1)</f>
+        <v/>
+      </c>
+      <c r="J18" s="5">
+        <f>IF(E18&lt;2,"积累中",IF(I18&gt;=0.01,"上涨",IF(I18&lt;=-0.01,"下降","平稳")))</f>
         <v/>
       </c>
     </row>
@@ -1999,7 +2108,7 @@
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="I5:I17">
+  <conditionalFormatting sqref="I5:I18">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="1">
       <formula>0.01</formula>
     </cfRule>
@@ -2114,7 +2223,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân / Vĩnh Tân</t>
+          <t>BAF / BAF</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -2134,7 +2243,7 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/ba-roi-heo-dac-biet-vinh-tan-400g-1-khay-63106</t>
+          <t>https://kingfoodmart.com/thit-heo/ba-roi-heo-baf-khay-300g-1-khay</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-08-30
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-30</t>
+          <t>越南猪肉零售价格日报｜2026-08-31</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 06:36。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 06:54。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>12条在售商品</t>
+          <t>11条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O16"/>
+  <dimension ref="A1:O15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-30</t>
+          <t>越南猪肉零售明细｜2026-08-31</t>
         </is>
       </c>
     </row>
@@ -1068,7 +1068,7 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g-ol341387</t>
         </is>
       </c>
     </row>
@@ -1364,12 +1364,12 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>肩肉</t>
+          <t>小排</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI Thịt Nạc vai heo (S)</t>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -1378,13 +1378,13 @@
         </is>
       </c>
       <c r="I13" s="7" t="n">
-        <v>440</v>
+        <v>431</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>74316</v>
+        <v>124085</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>168900</v>
+        <v>287900</v>
       </c>
       <c r="L13" s="7" t="n"/>
       <c r="M13" s="7">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="O13" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>
@@ -1430,12 +1430,12 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>小排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
+          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="I14" s="7" t="n">
-        <v>431</v>
+        <v>400</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>124085</v>
+        <v>81960</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>287900</v>
+        <v>204900</v>
       </c>
       <c r="L14" s="7" t="n"/>
       <c r="M14" s="7">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="O14" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
         </is>
       </c>
     </row>
@@ -1496,12 +1496,12 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -1510,13 +1510,13 @@
         </is>
       </c>
       <c r="I15" s="7" t="n">
-        <v>400</v>
+        <v>385</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>81960</v>
+        <v>76962</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>204900</v>
+        <v>199900</v>
       </c>
       <c r="L15" s="7" t="n"/>
       <c r="M15" s="7">
@@ -1529,72 +1529,6 @@
         </is>
       </c>
       <c r="O15" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="32" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>五花肉</t>
-        </is>
-      </c>
-      <c r="G16" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
-        </is>
-      </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I16" s="7" t="n">
-        <v>385</v>
-      </c>
-      <c r="J16" s="7" t="n">
-        <v>76962</v>
-      </c>
-      <c r="K16" s="7" t="n">
-        <v>199900</v>
-      </c>
-      <c r="L16" s="7" t="n"/>
-      <c r="M16" s="7">
-        <f>IF(L16&lt;&gt;"",L16,K16)</f>
-        <v/>
-      </c>
-      <c r="N16" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O16" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
@@ -1605,7 +1539,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M16">
+  <conditionalFormatting sqref="M5:M15">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1625,7 +1559,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1782,7 +1715,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>246667</v>
@@ -1824,7 +1757,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>199900</v>
@@ -1866,7 +1799,7 @@
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>287900</v>
@@ -1908,7 +1841,7 @@
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>204900</v>
@@ -1992,7 +1925,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>195000</v>
@@ -2034,7 +1967,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>138889</v>
@@ -2076,7 +2009,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>192100</v>
@@ -2118,7 +2051,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>138889</v>
@@ -2202,7 +2135,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>165000</v>
@@ -2244,7 +2177,7 @@
         </is>
       </c>
       <c r="E17" s="7" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F17" s="7" t="n">
         <v>190000</v>
@@ -2286,7 +2219,7 @@
         </is>
       </c>
       <c r="E18" s="7" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F18" s="7" t="n">
         <v>197500</v>
@@ -2510,7 +2443,7 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-09-01
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-08-31</t>
+          <t>越南猪肉零售价格日报｜2026-09-01</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 06:54。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 07:48。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>11条在售商品</t>
+          <t>10条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -632,7 +632,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>12组</t>
+          <t>0组</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-08-31</t>
+          <t>越南猪肉零售明细｜2026-09-01</t>
         </is>
       </c>
     </row>
@@ -1024,22 +1024,22 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
+          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1048,13 +1048,13 @@
         </is>
       </c>
       <c r="I8" s="7" t="n">
-        <v>900</v>
+        <v>200</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>125000</v>
+        <v>38000</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>138889</v>
+        <v>190000</v>
       </c>
       <c r="L8" s="7" t="n"/>
       <c r="M8" s="7">
@@ -1068,7 +1068,7 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g-ol341387</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
@@ -1090,22 +1090,22 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Thịt đùi Meatcool túi 900g</t>
+          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1114,13 +1114,13 @@
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>900</v>
+        <v>400</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>125000</v>
+        <v>79000</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>138889</v>
+        <v>197500</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
@@ -1134,7 +1134,7 @@
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g-ol341387</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
         </is>
       </c>
     </row>
@@ -1166,12 +1166,12 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
+          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -1183,10 +1183,10 @@
         <v>200</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>38000</v>
+        <v>33000</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>190000</v>
+        <v>165000</v>
       </c>
       <c r="L10" s="7" t="n"/>
       <c r="M10" s="7">
@@ -1200,44 +1200,44 @@
       </c>
       <c r="O10" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>肩肉</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
+          <t>MEATDELI Thịt Nạc vai heo (S)</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1246,13 +1246,13 @@
         </is>
       </c>
       <c r="I11" s="7" t="n">
-        <v>400</v>
+        <v>440</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>79000</v>
+        <v>74316</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>197500</v>
+        <v>168900</v>
       </c>
       <c r="L11" s="7" t="n"/>
       <c r="M11" s="7">
@@ -1261,49 +1261,49 @@
       </c>
       <c r="N11" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O11" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
+          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
         </is>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>小排</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="I12" s="7" t="n">
-        <v>200</v>
+        <v>431</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>33000</v>
+        <v>124085</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>165000</v>
+        <v>287900</v>
       </c>
       <c r="L12" s="7" t="n"/>
       <c r="M12" s="7">
@@ -1327,12 +1327,12 @@
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O12" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>
@@ -1364,12 +1364,12 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>小排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
+          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -1378,13 +1378,13 @@
         </is>
       </c>
       <c r="I13" s="7" t="n">
-        <v>431</v>
+        <v>400</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>124085</v>
+        <v>81960</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>287900</v>
+        <v>204900</v>
       </c>
       <c r="L13" s="7" t="n"/>
       <c r="M13" s="7">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="O13" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
         </is>
       </c>
     </row>
@@ -1430,12 +1430,12 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="I14" s="7" t="n">
-        <v>400</v>
+        <v>385</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>81960</v>
+        <v>76962</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>204900</v>
+        <v>199900</v>
       </c>
       <c r="L14" s="7" t="n"/>
       <c r="M14" s="7">
@@ -1463,72 +1463,6 @@
         </is>
       </c>
       <c r="O14" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>五花肉</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I15" s="7" t="n">
-        <v>385</v>
-      </c>
-      <c r="J15" s="7" t="n">
-        <v>76962</v>
-      </c>
-      <c r="K15" s="7" t="n">
-        <v>199900</v>
-      </c>
-      <c r="L15" s="7" t="n"/>
-      <c r="M15" s="7">
-        <f>IF(L15&lt;&gt;"",L15,K15)</f>
-        <v/>
-      </c>
-      <c r="N15" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O15" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
@@ -1539,7 +1473,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M15">
+  <conditionalFormatting sqref="M5:M14">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1558,7 +1492,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1570,7 +1503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1588,7 +1521,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>2026年8月同口径月度变化</t>
+          <t>2026年9月同口径月度变化</t>
         </is>
       </c>
     </row>
@@ -1664,7 +1597,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>五花肉</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -1676,13 +1609,13 @@
         <v>1</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>263333</v>
+        <v>246667</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>263333</v>
+        <v>246667</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>263333</v>
+        <v>246667</v>
       </c>
       <c r="I5" s="9">
         <f>IF(E5&lt;2,"",G5/F5-1)</f>
@@ -1696,35 +1629,35 @@
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>BAF</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>246667</v>
+        <v>199900</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>246667</v>
+        <v>199900</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>246667</v>
+        <v>199900</v>
       </c>
       <c r="I6" s="9">
         <f>IF(E6&lt;2,"",G6/F6-1)</f>
@@ -1748,7 +1681,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>五花肉</t>
+          <t>小排</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -1757,16 +1690,16 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>199900</v>
+        <v>287900</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>199900</v>
+        <v>287900</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>199900</v>
+        <v>287900</v>
       </c>
       <c r="I7" s="9">
         <f>IF(E7&lt;2,"",G7/F7-1)</f>
@@ -1790,7 +1723,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>小排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -1799,16 +1732,16 @@
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>287900</v>
+        <v>204900</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>287900</v>
+        <v>204900</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>287900</v>
+        <v>204900</v>
       </c>
       <c r="I8" s="9">
         <f>IF(E8&lt;2,"",G8/F8-1)</f>
@@ -1832,7 +1765,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>肩肉</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -1841,16 +1774,16 @@
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>204900</v>
+        <v>168900</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>204900</v>
+        <v>168900</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>204900</v>
+        <v>168900</v>
       </c>
       <c r="I9" s="9">
         <f>IF(E9&lt;2,"",G9/F9-1)</f>
@@ -1864,35 +1797,35 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>WinMart</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>MEATDeli</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>肩肉</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>WinMart默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="E10" s="7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>168900</v>
+        <v>175555</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>168900</v>
+        <v>175555</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>168900</v>
+        <v>175555</v>
       </c>
       <c r="I10" s="9">
         <f>IF(E10&lt;2,"",G10/F10-1)</f>
@@ -1916,7 +1849,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>五花肉</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -1925,16 +1858,16 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>195000</v>
+        <v>192100</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>175555</v>
+        <v>192100</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>195000</v>
+        <v>192100</v>
       </c>
       <c r="I11" s="9">
         <f>IF(E11&lt;2,"",G11/F11-1)</f>
@@ -1953,7 +1886,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -1967,16 +1900,16 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>138889</v>
+        <v>165000</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>138889</v>
+        <v>165000</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>138889</v>
+        <v>165000</v>
       </c>
       <c r="I12" s="9">
         <f>IF(E12&lt;2,"",G12/F12-1)</f>
@@ -1995,7 +1928,7 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
@@ -2009,16 +1942,16 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>192100</v>
+        <v>190000</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>192100</v>
+        <v>190000</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>192100</v>
+        <v>190000</v>
       </c>
       <c r="I13" s="9">
         <f>IF(E13&lt;2,"",G13/F13-1)</f>
@@ -2037,7 +1970,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -2051,16 +1984,16 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>138889</v>
+        <v>197500</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>138889</v>
+        <v>197500</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>138889</v>
+        <v>197500</v>
       </c>
       <c r="I14" s="9">
         <f>IF(E14&lt;2,"",G14/F14-1)</f>
@@ -2068,174 +2001,6 @@
       </c>
       <c r="J14" s="5">
         <f>IF(E14&lt;2,"积累中",IF(I14&gt;=0.01,"上涨",IF(I14&lt;=-0.01,"下降","平稳")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Kingfoodmart</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Vĩnh Tân</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>五花肉</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" s="7" t="n">
-        <v>222500</v>
-      </c>
-      <c r="G15" s="7" t="n">
-        <v>222500</v>
-      </c>
-      <c r="H15" s="7" t="n">
-        <v>222500</v>
-      </c>
-      <c r="I15" s="9">
-        <f>IF(E15&lt;2,"",G15/F15-1)</f>
-        <v/>
-      </c>
-      <c r="J15" s="5">
-        <f>IF(E15&lt;2,"积累中",IF(I15&gt;=0.01,"上涨",IF(I15&lt;=-0.01,"下降","平稳")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Kingfoodmart</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Vĩnh Tân</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>后腿肉</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
-        </is>
-      </c>
-      <c r="E16" s="7" t="n">
-        <v>22</v>
-      </c>
-      <c r="F16" s="7" t="n">
-        <v>165000</v>
-      </c>
-      <c r="G16" s="7" t="n">
-        <v>165000</v>
-      </c>
-      <c r="H16" s="7" t="n">
-        <v>165000</v>
-      </c>
-      <c r="I16" s="9">
-        <f>IF(E16&lt;2,"",G16/F16-1)</f>
-        <v/>
-      </c>
-      <c r="J16" s="5">
-        <f>IF(E16&lt;2,"积累中",IF(I16&gt;=0.01,"上涨",IF(I16&lt;=-0.01,"下降","平稳")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>Kingfoodmart</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Vĩnh Tân</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>梅花肉</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="n">
-        <v>29</v>
-      </c>
-      <c r="F17" s="7" t="n">
-        <v>190000</v>
-      </c>
-      <c r="G17" s="7" t="n">
-        <v>190000</v>
-      </c>
-      <c r="H17" s="7" t="n">
-        <v>190000</v>
-      </c>
-      <c r="I17" s="9">
-        <f>IF(E17&lt;2,"",G17/F17-1)</f>
-        <v/>
-      </c>
-      <c r="J17" s="5">
-        <f>IF(E17&lt;2,"积累中",IF(I17&gt;=0.01,"上涨",IF(I17&lt;=-0.01,"下降","平稳")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Kingfoodmart</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Vĩnh Tân</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>猪排</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="n">
-        <v>29</v>
-      </c>
-      <c r="F18" s="7" t="n">
-        <v>197500</v>
-      </c>
-      <c r="G18" s="7" t="n">
-        <v>197500</v>
-      </c>
-      <c r="H18" s="7" t="n">
-        <v>197500</v>
-      </c>
-      <c r="I18" s="9">
-        <f>IF(E18&lt;2,"",G18/F18-1)</f>
-        <v/>
-      </c>
-      <c r="J18" s="5">
-        <f>IF(E18&lt;2,"积累中",IF(I18&gt;=0.01,"上涨",IF(I18&lt;=-0.01,"下降","平稳")))</f>
         <v/>
       </c>
     </row>
@@ -2244,7 +2009,7 @@
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="I5:I18">
+  <conditionalFormatting sqref="I5:I14">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="1">
       <formula>0.01</formula>
     </cfRule>
@@ -2443,7 +2208,7 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-09-02
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-09-02</t>
+          <t>越南猪肉零售价格日报｜2026-09-03</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 06:34。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 06:33。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>11条在售商品</t>
+          <t>10条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -632,7 +632,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>9组</t>
+          <t>11组</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-09-02</t>
+          <t>越南猪肉零售明细｜2026-09-03</t>
         </is>
       </c>
     </row>
@@ -1465,72 +1465,6 @@
       <c r="O14" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>五花肉</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I15" s="7" t="n">
-        <v>385</v>
-      </c>
-      <c r="J15" s="7" t="n">
-        <v>76962</v>
-      </c>
-      <c r="K15" s="7" t="n">
-        <v>199900</v>
-      </c>
-      <c r="L15" s="7" t="n"/>
-      <c r="M15" s="7">
-        <f>IF(L15&lt;&gt;"",L15,K15)</f>
-        <v/>
-      </c>
-      <c r="N15" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O15" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
       </c>
     </row>
@@ -1539,7 +1473,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M15">
+  <conditionalFormatting sqref="M5:M14">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1558,7 +1492,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1673,7 +1606,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1757,7 +1690,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1799,7 +1732,7 @@
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>204900</v>
@@ -1883,7 +1816,7 @@
         </is>
       </c>
       <c r="E10" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F10" s="7" t="n">
         <v>175555</v>
@@ -1925,7 +1858,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1967,7 +1900,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -2009,7 +1942,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -2051,7 +1984,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>165000</v>
@@ -2093,7 +2026,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
@@ -2135,7 +2068,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-09-03
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-09-03</t>
+          <t>越南猪肉零售价格日报｜2026-09-04</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 06:33。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 06:40。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-09-03</t>
+          <t>越南猪肉零售明细｜2026-09-04</t>
         </is>
       </c>
     </row>
@@ -1430,12 +1430,12 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="I14" s="7" t="n">
-        <v>400</v>
+        <v>385</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>81960</v>
+        <v>76962</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>204900</v>
+        <v>199900</v>
       </c>
       <c r="L14" s="7" t="n"/>
       <c r="M14" s="7">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="O14" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
+          <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
       </c>
     </row>
@@ -1606,7 +1606,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1648,7 +1648,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1690,7 +1690,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1816,7 +1816,7 @@
         </is>
       </c>
       <c r="E10" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F10" s="7" t="n">
         <v>175555</v>
@@ -1858,7 +1858,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1900,7 +1900,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -1942,7 +1942,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -1984,7 +1984,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>165000</v>
@@ -2026,7 +2026,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
@@ -2068,7 +2068,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-09-04
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-09-04</t>
+          <t>越南猪肉零售价格日报｜2026-09-05</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 06:40。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 06:21。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>10条在售商品</t>
+          <t>12条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -632,7 +632,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>11组</t>
+          <t>12组</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:O16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-09-04</t>
+          <t>越南猪肉零售明细｜2026-09-05</t>
         </is>
       </c>
     </row>
@@ -1364,12 +1364,12 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>小排</t>
+          <t>肩肉</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
+          <t>MEATDELI Thịt Nạc vai heo (S)</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -1378,13 +1378,13 @@
         </is>
       </c>
       <c r="I13" s="7" t="n">
-        <v>431</v>
+        <v>440</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>124085</v>
+        <v>74316</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>287900</v>
+        <v>168900</v>
       </c>
       <c r="L13" s="7" t="n"/>
       <c r="M13" s="7">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="O13" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
         </is>
       </c>
     </row>
@@ -1430,12 +1430,12 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>五花肉</t>
+          <t>小排</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="I14" s="7" t="n">
-        <v>385</v>
+        <v>431</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>76962</v>
+        <v>124085</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>199900</v>
+        <v>287900</v>
       </c>
       <c r="L14" s="7" t="n"/>
       <c r="M14" s="7">
@@ -1463,6 +1463,138 @@
         </is>
       </c>
       <c r="O14" s="8" t="inlineStr">
+        <is>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>全国渠道</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>WinMart默认门店（待固定城市）</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>WinMart</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Masan</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>MEATDeli</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>梅花肉</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>冷鲜</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>400</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>81960</v>
+      </c>
+      <c r="K15" s="7" t="n">
+        <v>204900</v>
+      </c>
+      <c r="L15" s="7" t="n"/>
+      <c r="M15" s="7">
+        <f>IF(L15&lt;&gt;"",L15,K15)</f>
+        <v/>
+      </c>
+      <c r="N15" s="5" t="inlineStr">
+        <is>
+          <t>中：官方交易页，但尚未固定配送门店</t>
+        </is>
+      </c>
+      <c r="O15" s="8" t="inlineStr">
+        <is>
+          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="32" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>全国渠道</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>WinMart默认门店（待固定城市）</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>WinMart</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Masan</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>MEATDeli</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>五花肉</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>冷鲜</t>
+        </is>
+      </c>
+      <c r="I16" s="7" t="n">
+        <v>385</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>76962</v>
+      </c>
+      <c r="K16" s="7" t="n">
+        <v>199900</v>
+      </c>
+      <c r="L16" s="7" t="n"/>
+      <c r="M16" s="7">
+        <f>IF(L16&lt;&gt;"",L16,K16)</f>
+        <v/>
+      </c>
+      <c r="N16" s="5" t="inlineStr">
+        <is>
+          <t>中：官方交易页，但尚未固定配送门店</t>
+        </is>
+      </c>
+      <c r="O16" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
@@ -1473,7 +1605,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M14">
+  <conditionalFormatting sqref="M5:M16">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1492,6 +1624,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1606,7 +1740,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1648,7 +1782,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1690,7 +1824,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1732,7 +1866,7 @@
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>204900</v>
@@ -1774,7 +1908,7 @@
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>168900</v>
@@ -1816,7 +1950,7 @@
         </is>
       </c>
       <c r="E10" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F10" s="7" t="n">
         <v>175555</v>
@@ -1858,7 +1992,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1900,7 +2034,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -1942,7 +2076,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -1984,7 +2118,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>165000</v>
@@ -2026,7 +2160,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
@@ -2068,7 +2202,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>
@@ -2292,7 +2426,7 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-09-05
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-09-05</t>
+          <t>越南猪肉零售价格日报｜2026-09-06</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 06:21。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 06:19。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>12条在售商品</t>
+          <t>11条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O16"/>
+  <dimension ref="A1:O15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-09-05</t>
+          <t>越南猪肉零售明细｜2026-09-06</t>
         </is>
       </c>
     </row>
@@ -1034,12 +1034,12 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
+          <t>Thịt đùi Meatcool túi 900g</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1068,7 +1068,7 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -1100,12 +1100,12 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Thịt đùi Meatcool túi 900g</t>
+          <t>Cốt lết heo Meatcool khay 300g</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1114,13 +1114,13 @@
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>900</v>
+        <v>300</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>125000</v>
+        <v>35000</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>138889</v>
+        <v>116667</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
@@ -1134,7 +1134,7 @@
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/sap-mo-ban-cot-let-heo-meatcool-khay-300g-ol344147</t>
         </is>
       </c>
     </row>
@@ -1273,37 +1273,37 @@
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>肩肉</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
+          <t>MEATDELI Thịt Nạc vai heo (S)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="I12" s="7" t="n">
-        <v>200</v>
+        <v>440</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>33000</v>
+        <v>74316</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>165000</v>
+        <v>168900</v>
       </c>
       <c r="L12" s="7" t="n"/>
       <c r="M12" s="7">
@@ -1327,12 +1327,12 @@
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O12" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
+          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
         </is>
       </c>
     </row>
@@ -1364,12 +1364,12 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>肩肉</t>
+          <t>小排</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI Thịt Nạc vai heo (S)</t>
+          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -1378,13 +1378,13 @@
         </is>
       </c>
       <c r="I13" s="7" t="n">
-        <v>440</v>
+        <v>431</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>74316</v>
+        <v>124085</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>168900</v>
+        <v>287900</v>
       </c>
       <c r="L13" s="7" t="n"/>
       <c r="M13" s="7">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="O13" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>
@@ -1430,12 +1430,12 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>小排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI [PRE] Thịt Sườn thăn (sườn non) (S)</t>
+          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="I14" s="7" t="n">
-        <v>431</v>
+        <v>400</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>124085</v>
+        <v>81960</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>287900</v>
+        <v>204900</v>
       </c>
       <c r="L14" s="7" t="n"/>
       <c r="M14" s="7">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="O14" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
         </is>
       </c>
     </row>
@@ -1496,12 +1496,12 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
@@ -1510,13 +1510,13 @@
         </is>
       </c>
       <c r="I15" s="7" t="n">
-        <v>400</v>
+        <v>385</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>81960</v>
+        <v>76962</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>204900</v>
+        <v>199900</v>
       </c>
       <c r="L15" s="7" t="n"/>
       <c r="M15" s="7">
@@ -1529,72 +1529,6 @@
         </is>
       </c>
       <c r="O15" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="32" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>五花肉</t>
-        </is>
-      </c>
-      <c r="G16" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
-        </is>
-      </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I16" s="7" t="n">
-        <v>385</v>
-      </c>
-      <c r="J16" s="7" t="n">
-        <v>76962</v>
-      </c>
-      <c r="K16" s="7" t="n">
-        <v>199900</v>
-      </c>
-      <c r="L16" s="7" t="n"/>
-      <c r="M16" s="7">
-        <f>IF(L16&lt;&gt;"",L16,K16)</f>
-        <v/>
-      </c>
-      <c r="N16" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O16" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
@@ -1605,7 +1539,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M16">
+  <conditionalFormatting sqref="M5:M15">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1625,7 +1559,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1740,7 +1673,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1782,7 +1715,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1824,7 +1757,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1866,7 +1799,7 @@
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>204900</v>
@@ -1908,7 +1841,7 @@
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>168900</v>
@@ -1950,7 +1883,7 @@
         </is>
       </c>
       <c r="E10" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F10" s="7" t="n">
         <v>175555</v>
@@ -1992,7 +1925,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -2034,7 +1967,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -2076,13 +2009,13 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>138889</v>
+        <v>116667</v>
       </c>
       <c r="H13" s="7" t="n">
         <v>138889</v>
@@ -2160,7 +2093,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
@@ -2202,7 +2135,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-09-06
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-09-06</t>
+          <t>越南猪肉零售价格日报｜2026-09-07</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 06:19。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 06:10。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-09-06</t>
+          <t>越南猪肉零售明细｜2026-09-07</t>
         </is>
       </c>
     </row>
@@ -914,16 +914,16 @@
         </is>
       </c>
       <c r="I6" s="7" t="n">
-        <v>450</v>
+        <v>400</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>112050</v>
+        <v>99600</v>
       </c>
       <c r="K6" s="7" t="n">
         <v>249000</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>175555</v>
+        <v>207250</v>
       </c>
       <c r="M6" s="7">
         <f>IF(L6&lt;&gt;"",L6,K6)</f>
@@ -1034,12 +1034,12 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Thịt đùi Meatcool túi 900g</t>
+          <t>Cốt lết heo Meatcool khay 300g</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1048,13 +1048,13 @@
         </is>
       </c>
       <c r="I8" s="7" t="n">
-        <v>900</v>
+        <v>300</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>125000</v>
+        <v>35000</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>138889</v>
+        <v>116667</v>
       </c>
       <c r="L8" s="7" t="n"/>
       <c r="M8" s="7">
@@ -1068,7 +1068,7 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/cot-let-heo-meatcool-khay-300g</t>
         </is>
       </c>
     </row>
@@ -1090,22 +1090,22 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Cốt lết heo Meatcool khay 300g</t>
+          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1114,13 +1114,13 @@
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>35000</v>
+        <v>38000</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>116667</v>
+        <v>190000</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
@@ -1134,7 +1134,7 @@
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/sap-mo-ban-cot-let-heo-meatcool-khay-300g-ol344147</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
@@ -1166,12 +1166,12 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
+          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -1180,13 +1180,13 @@
         </is>
       </c>
       <c r="I10" s="7" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>38000</v>
+        <v>79000</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>190000</v>
+        <v>197500</v>
       </c>
       <c r="L10" s="7" t="n"/>
       <c r="M10" s="7">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="O10" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
         </is>
       </c>
     </row>
@@ -1232,12 +1232,12 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
+          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1246,13 +1246,13 @@
         </is>
       </c>
       <c r="I11" s="7" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>79000</v>
+        <v>33000</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>197500</v>
+        <v>165000</v>
       </c>
       <c r="L11" s="7" t="n"/>
       <c r="M11" s="7">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="O11" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
@@ -1673,7 +1673,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1715,7 +1715,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1757,7 +1757,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1799,7 +1799,7 @@
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>204900</v>
@@ -1841,7 +1841,7 @@
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>168900</v>
@@ -1883,13 +1883,13 @@
         </is>
       </c>
       <c r="E10" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F10" s="7" t="n">
         <v>175555</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>175555</v>
+        <v>207250</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>175555</v>
@@ -1967,7 +1967,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -2009,7 +2009,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -2051,7 +2051,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>165000</v>
@@ -2093,7 +2093,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
@@ -2135,7 +2135,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-09-07
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-09-07</t>
+          <t>越南猪肉零售价格日报｜2026-09-08</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 06:10。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 06:46。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-09-07</t>
+          <t>越南猪肉零售明细｜2026-09-08</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
         <v>249000</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>207250</v>
+        <v>197500</v>
       </c>
       <c r="M6" s="7">
         <f>IF(L6&lt;&gt;"",L6,K6)</f>
@@ -1034,12 +1034,12 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Cốt lết heo Meatcool khay 300g</t>
+          <t>Thịt đùi Meatcool túi 900g</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1048,13 +1048,13 @@
         </is>
       </c>
       <c r="I8" s="7" t="n">
-        <v>300</v>
+        <v>900</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>35000</v>
+        <v>125000</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>116667</v>
+        <v>138889</v>
       </c>
       <c r="L8" s="7" t="n"/>
       <c r="M8" s="7">
@@ -1068,7 +1068,7 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/cot-let-heo-meatcool-khay-300g</t>
+          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -1090,22 +1090,22 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
+          <t>Cốt lết heo Meatcool khay 300g</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1114,13 +1114,13 @@
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>38000</v>
+        <v>35000</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>190000</v>
+        <v>116667</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
@@ -1134,7 +1134,7 @@
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
+          <t>https://kingfoodmart.com/thit-heo/cot-let-heo-meatcool-khay-300g</t>
         </is>
       </c>
     </row>
@@ -1166,12 +1166,12 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
+          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -1180,13 +1180,13 @@
         </is>
       </c>
       <c r="I10" s="7" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>79000</v>
+        <v>38000</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>197500</v>
+        <v>190000</v>
       </c>
       <c r="L10" s="7" t="n"/>
       <c r="M10" s="7">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="O10" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
@@ -1232,12 +1232,12 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
+          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1246,13 +1246,13 @@
         </is>
       </c>
       <c r="I11" s="7" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>33000</v>
+        <v>79000</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>165000</v>
+        <v>197500</v>
       </c>
       <c r="L11" s="7" t="n"/>
       <c r="M11" s="7">
@@ -1266,44 +1266,44 @@
       </c>
       <c r="O11" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
         </is>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>全国渠道</t>
+          <t>南部</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>WinMart默认门店（待固定城市）</t>
+          <t>胡志明市/Kingfoodmart默认门店</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>WinMart</t>
+          <t>Kingfoodmart</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Masan</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>MEATDeli</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>肩肉</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI Thịt Nạc vai heo (S)</t>
+          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1312,13 +1312,13 @@
         </is>
       </c>
       <c r="I12" s="7" t="n">
-        <v>440</v>
+        <v>200</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>74316</v>
+        <v>33000</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>168900</v>
+        <v>165000</v>
       </c>
       <c r="L12" s="7" t="n"/>
       <c r="M12" s="7">
@@ -1327,12 +1327,12 @@
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
+          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
         </is>
       </c>
       <c r="O12" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
@@ -1673,7 +1673,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1715,7 +1715,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1757,7 +1757,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1799,7 +1799,7 @@
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F8" s="7" t="n">
         <v>204900</v>
@@ -1883,13 +1883,13 @@
         </is>
       </c>
       <c r="E10" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F10" s="7" t="n">
         <v>175555</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>207250</v>
+        <v>197500</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>175555</v>
@@ -1925,7 +1925,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1967,7 +1967,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -2009,7 +2009,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -2051,7 +2051,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>165000</v>
@@ -2093,7 +2093,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
@@ -2135,7 +2135,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
+          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-09-08
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-09-08</t>
+          <t>越南猪肉零售价格日报｜2026-09-09</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 06:46。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 06:40。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>11条在售商品</t>
+          <t>10条在售商品</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-09-08</t>
+          <t>越南猪肉零售明细｜2026-09-09</t>
         </is>
       </c>
     </row>
@@ -1430,12 +1430,12 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>五花肉</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>MEATDELI Thịt Nạc dăm heo (Thịt Nạc vai) (S)</t>
+          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
@@ -1444,13 +1444,13 @@
         </is>
       </c>
       <c r="I14" s="7" t="n">
-        <v>400</v>
+        <v>385</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>81960</v>
+        <v>76962</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>204900</v>
+        <v>199900</v>
       </c>
       <c r="L14" s="7" t="n"/>
       <c r="M14" s="7">
@@ -1463,72 +1463,6 @@
         </is>
       </c>
       <c r="O14" s="8" t="inlineStr">
-        <is>
-          <t>https://winmart.vn/products/meat-deli-nac-dam-heo--s10617957</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>全国渠道</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>WinMart默认门店（待固定城市）</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>WinMart</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Masan</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>MEATDeli</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>五花肉</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>MEATDELI Thịt Ba Rọi heo (S)</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>冷鲜</t>
-        </is>
-      </c>
-      <c r="I15" s="7" t="n">
-        <v>385</v>
-      </c>
-      <c r="J15" s="7" t="n">
-        <v>76962</v>
-      </c>
-      <c r="K15" s="7" t="n">
-        <v>199900</v>
-      </c>
-      <c r="L15" s="7" t="n"/>
-      <c r="M15" s="7">
-        <f>IF(L15&lt;&gt;"",L15,K15)</f>
-        <v/>
-      </c>
-      <c r="N15" s="5" t="inlineStr">
-        <is>
-          <t>中：官方交易页，但尚未固定配送门店</t>
-        </is>
-      </c>
-      <c r="O15" s="8" t="inlineStr">
         <is>
           <t>https://winmart.vn/products/meat-deli-ba-roi-heo--s10617959</t>
         </is>
@@ -1539,7 +1473,7 @@
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
-  <conditionalFormatting sqref="M5:M15">
+  <conditionalFormatting sqref="M5:M14">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>150000</formula>
     </cfRule>
@@ -1558,7 +1492,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1673,7 +1606,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1715,7 +1648,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1757,7 +1690,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1883,7 +1816,7 @@
         </is>
       </c>
       <c r="E10" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F10" s="7" t="n">
         <v>175555</v>
@@ -1925,7 +1858,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1967,7 +1900,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -2009,7 +1942,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -2018,7 +1951,7 @@
         <v>116667</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>138889</v>
+        <v>127778</v>
       </c>
       <c r="I13" s="9">
         <f>IF(E13&lt;2,"",G13/F13-1)</f>
@@ -2051,7 +1984,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>165000</v>
@@ -2093,7 +2026,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
@@ -2135,7 +2068,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-09-09
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-09-09</t>
+          <t>越南猪肉零售价格日报｜2026-09-10</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 06:40。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 06:30。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-09-09</t>
+          <t>越南猪肉零售明细｜2026-09-10</t>
         </is>
       </c>
     </row>
@@ -890,22 +890,22 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>BAF</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>BAF</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>五花肉</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Ba rọi heo Meatcool 350-450g</t>
+          <t>Nạc dăm heo BAF khay 300g</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -914,17 +914,15 @@
         </is>
       </c>
       <c r="I6" s="7" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>99600</v>
+        <v>74000</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>249000</v>
-      </c>
-      <c r="L6" s="7" t="n">
-        <v>197500</v>
-      </c>
+        <v>246667</v>
+      </c>
+      <c r="L6" s="7" t="n"/>
       <c r="M6" s="7">
         <f>IF(L6&lt;&gt;"",L6,K6)</f>
         <v/>
@@ -936,7 +934,7 @@
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/ba-roi-heo-meatcool-400g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
         </is>
       </c>
     </row>
@@ -958,22 +956,22 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>BAF</t>
+          <t>GREENFEED</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>BAF</t>
+          <t>Meatcool</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo BAF khay 300g</t>
+          <t>Cốt lết Meatcool 9-10 miếng/túi 900g</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -982,13 +980,13 @@
         </is>
       </c>
       <c r="I7" s="7" t="n">
-        <v>300</v>
+        <v>900</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>74000</v>
+        <v>125000</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>246667</v>
+        <v>138889</v>
       </c>
       <c r="L7" s="7" t="n"/>
       <c r="M7" s="7">
@@ -1002,7 +1000,7 @@
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-baf-khay-300g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -1068,7 +1066,7 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/sap-mo-ban-thit-dui-meatcool-tui-900g-ol341387</t>
         </is>
       </c>
     </row>
@@ -1090,22 +1088,22 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>GREENFEED</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Meatcool</t>
+          <t>Vĩnh Tân</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>梅花肉</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Cốt lết heo Meatcool khay 300g</t>
+          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1114,13 +1112,13 @@
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>35000</v>
+        <v>38000</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>116667</v>
+        <v>190000</v>
       </c>
       <c r="L9" s="7" t="n"/>
       <c r="M9" s="7">
@@ -1134,7 +1132,7 @@
       </c>
       <c r="O9" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/cot-let-heo-meatcool-khay-300g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
@@ -1166,12 +1164,12 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>梅花肉</t>
+          <t>猪排</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Nạc dăm heo Vĩnh Tân khay 200g</t>
+          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -1180,13 +1178,13 @@
         </is>
       </c>
       <c r="I10" s="7" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>38000</v>
+        <v>79000</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>190000</v>
+        <v>197500</v>
       </c>
       <c r="L10" s="7" t="n"/>
       <c r="M10" s="7">
@@ -1200,7 +1198,7 @@
       </c>
       <c r="O10" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dam-heo-vinh-tan-khay-200g</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
         </is>
       </c>
     </row>
@@ -1232,12 +1230,12 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>猪排</t>
+          <t>后腿肉</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Nạc cốt lết cắt Vĩnh Tân khay 400g</t>
+          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1246,13 +1244,13 @@
         </is>
       </c>
       <c r="I11" s="7" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>79000</v>
+        <v>33000</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>197500</v>
+        <v>165000</v>
       </c>
       <c r="L11" s="7" t="n"/>
       <c r="M11" s="7">
@@ -1266,44 +1264,44 @@
       </c>
       <c r="O11" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-cot-let-cat-vinh-tan-khay-400g-1-khay</t>
+          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
         </is>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>南部</t>
+          <t>全国渠道</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>胡志明市/Kingfoodmart默认门店</t>
+          <t>WinMart默认门店（待固定城市）</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Kingfoodmart</t>
+          <t>WinMart</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>Masan</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Vĩnh Tân</t>
+          <t>MEATDeli</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>后腿肉</t>
+          <t>肩肉</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Nạc đùi heo cắt xào Vĩnh Tân khay 200g</t>
+          <t>MEATDELI Thịt Nạc vai heo (S)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1312,13 +1310,13 @@
         </is>
       </c>
       <c r="I12" s="7" t="n">
-        <v>200</v>
+        <v>440</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>33000</v>
+        <v>74316</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>165000</v>
+        <v>168900</v>
       </c>
       <c r="L12" s="7" t="n"/>
       <c r="M12" s="7">
@@ -1327,12 +1325,12 @@
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>中：交易页含价格/重量/库存，但尚未锁定具体门店</t>
+          <t>中：官方交易页，但尚未固定配送门店</t>
         </is>
       </c>
       <c r="O12" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/nac-dui-heo-cat-xao-vinh-tan-khay-200g</t>
+          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
         </is>
       </c>
     </row>
@@ -1606,7 +1604,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1648,7 +1646,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1690,7 +1688,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1774,7 +1772,7 @@
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>168900</v>
@@ -1858,7 +1856,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1900,7 +1898,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -1942,16 +1940,16 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>116667</v>
+        <v>138889</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>127778</v>
+        <v>138889</v>
       </c>
       <c r="I13" s="9">
         <f>IF(E13&lt;2,"",G13/F13-1)</f>
@@ -1984,7 +1982,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>165000</v>
@@ -2026,7 +2024,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
@@ -2068,7 +2066,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>
@@ -2292,7 +2290,7 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>https://winmart.vn/products/meat-deli-sig-suon-than-suon-non--s10281593</t>
+          <t>https://winmart.vn/products/meat-deli-nac-vai-heo-s--s10140279</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-09-10
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-09-10</t>
+          <t>越南猪肉零售价格日报｜2026-09-11</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 06:30。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 06:24。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-09-10</t>
+          <t>越南猪肉零售明细｜2026-09-11</t>
         </is>
       </c>
     </row>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="O8" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/sap-mo-ban-thit-dui-meatcool-tui-900g-ol341387</t>
+          <t>https://kingfoodmart.com/thit-heo/thit-dui-meatcool-tui-900g</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1646,7 +1646,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1688,7 +1688,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1772,7 +1772,7 @@
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>168900</v>
@@ -1856,7 +1856,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1898,7 +1898,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -1940,7 +1940,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -1982,7 +1982,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>165000</v>
@@ -2024,7 +2024,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
@@ -2066,7 +2066,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>

</xml_diff>

<commit_message>
publish pork retail Excel 2026-09-11
</commit_message>
<xml_diff>
--- a/reports/越南猪肉零售价格日报_最新.xlsx
+++ b/reports/越南猪肉零售价格日报_最新.xlsx
@@ -547,14 +547,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售价格日报｜2026-09-11</t>
+          <t>越南猪肉零售价格日报｜2026-09-12</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>采集时间：越南时间 06:24。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
+          <t>采集时间：越南时间 06:32。所有商品售价均统一折算为 VND/kg；常规价和促销价分别保留。</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南猪肉零售明细｜2026-09-11</t>
+          <t>越南猪肉零售明细｜2026-09-12</t>
         </is>
       </c>
     </row>
@@ -1000,7 +1000,7 @@
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g</t>
+          <t>https://kingfoodmart.com/thit-heo/cot-let-meatcool-tui-900g-ol341387</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F5" s="7" t="n">
         <v>246667</v>
@@ -1646,7 +1646,7 @@
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F6" s="7" t="n">
         <v>199900</v>
@@ -1688,7 +1688,7 @@
         </is>
       </c>
       <c r="E7" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F7" s="7" t="n">
         <v>287900</v>
@@ -1772,7 +1772,7 @@
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>168900</v>
@@ -1856,7 +1856,7 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F11" s="7" t="n">
         <v>138889</v>
@@ -1898,7 +1898,7 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F12" s="7" t="n">
         <v>192100</v>
@@ -1940,7 +1940,7 @@
         </is>
       </c>
       <c r="E13" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F13" s="7" t="n">
         <v>138889</v>
@@ -1982,7 +1982,7 @@
         </is>
       </c>
       <c r="E14" s="7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F14" s="7" t="n">
         <v>165000</v>
@@ -2024,7 +2024,7 @@
         </is>
       </c>
       <c r="E15" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>190000</v>
@@ -2066,7 +2066,7 @@
         </is>
       </c>
       <c r="E16" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F16" s="7" t="n">
         <v>197500</v>

</xml_diff>